<commit_message>
Fix LBOMODEL4 xlsx so Excel can open it
Prior openpyxl resave wrote absolute /xl/ relationship targets and
orphan chart/comment parts Excel rejects. Rebuild strips charts/drawings
and rewrites relative OOXML relationships.

Co-authored-by: vengeanceaiUSC <vengeanceaiUSC@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/vengeanceaiUSC_LBOMODEL4.xlsx
+++ b/vengeanceaiUSC_LBOMODEL4.xlsx
@@ -18,10 +18,6 @@
     <sheet name="Shares" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="52wkHL" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId12"/>
-    <externalReference r:id="rId13"/>
-  </externalReferences>
   <definedNames>
     <definedName name="CIQWBGuid" hidden="1">"a611639b-bab1-425e-aaa5-008c326fdfdb"</definedName>
     <definedName name="Inv_Cap">[1]Results!$E$182:$AD$182</definedName>
@@ -68,7 +64,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="87">
+  <numFmts count="85">
     <numFmt numFmtId="164" formatCode="#,##0.0_);\(#,##0.0\);@_)"/>
     <numFmt numFmtId="165" formatCode="0.0%_);\(0.0%\);@_)"/>
     <numFmt numFmtId="166" formatCode="0\A;[Red]0\A"/>
@@ -97,65 +93,63 @@
     <numFmt numFmtId="189" formatCode="0.000%"/>
     <numFmt numFmtId="190" formatCode="#,##0.0"/>
     <numFmt numFmtId="191" formatCode="0.00\x"/>
-    <numFmt numFmtId="192" formatCode="YYYY-MM-DD"/>
-    <numFmt numFmtId="193" formatCode="0.000"/>
-    <numFmt numFmtId="194" formatCode="0.0000"/>
-    <numFmt numFmtId="195" formatCode="0.0x"/>
-    <numFmt numFmtId="196" formatCode="0.00x"/>
-    <numFmt numFmtId="197" formatCode="#,##0.00_);\(#,##0\)"/>
-    <numFmt numFmtId="198" formatCode="#,##0.0%_);\(#,##0.0%\)"/>
-    <numFmt numFmtId="199" formatCode="0.0\ \x"/>
-    <numFmt numFmtId="200" formatCode="#,##0.00\ ;\(#,##0.00\)"/>
-    <numFmt numFmtId="201" formatCode="&quot;$&quot;#,##0.00\ ;\(&quot;$&quot;#,##0.00\)"/>
-    <numFmt numFmtId="202" formatCode="0.0%_);\(0.0%\)"/>
-    <numFmt numFmtId="203" formatCode="0.000\ \x&quot;rate&quot;"/>
-    <numFmt numFmtId="204" formatCode="#,##0.000_);[Red]\(#,##0.000\)"/>
-    <numFmt numFmtId="205" formatCode="0.00_);\(0.00\);0.00"/>
-    <numFmt numFmtId="206" formatCode="\C&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
-    <numFmt numFmtId="207" formatCode="#,##0%_);\(#,##0.0%\)"/>
-    <numFmt numFmtId="208" formatCode="_(* #,##0.00000000_);_(* \(#,##0.00000000\);_(* &quot;-&quot;?_);_(@_)"/>
-    <numFmt numFmtId="209" formatCode="mmm\-d\-yyyy"/>
-    <numFmt numFmtId="210" formatCode="mmm\-yyyy"/>
-    <numFmt numFmtId="211" formatCode="yyyy"/>
-    <numFmt numFmtId="212" formatCode="0.00\x&quot;rate&quot;"/>
-    <numFmt numFmtId="213" formatCode="0.0&quot;  &quot;"/>
-    <numFmt numFmtId="214" formatCode="&quot;$&quot;#,##0.0\ ;[Red]\(&quot;$&quot;#,##0\)"/>
-    <numFmt numFmtId="215" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;?_);_(@_)"/>
-    <numFmt numFmtId="216" formatCode="&quot;$&quot;#,##0.000_);[Red]\(&quot;$&quot;#,##0.000\)"/>
-    <numFmt numFmtId="217" formatCode="&quot;$&quot;#,##0.00&quot;A&quot;;[Red]\(&quot;$&quot;#,##0.00\)&quot;A&quot;"/>
-    <numFmt numFmtId="218" formatCode="#,##0.0\ ;[Red]\(&quot;$&quot;#,##0\)"/>
-    <numFmt numFmtId="219" formatCode="&quot;$&quot;#,##0.00&quot;E&quot;;[Red]\(&quot;$&quot;#,##0.00\)&quot;E&quot;"/>
-    <numFmt numFmtId="220" formatCode="_([$€-2]* #,##0.00_);_([$€-2]* \(#,##0.00\);_([$€-2]* &quot;-&quot;??_)"/>
-    <numFmt numFmtId="221" formatCode="#,##0.00;\(#,##0.00\)"/>
-    <numFmt numFmtId="222" formatCode=".%\,\(0.0%%;\t"/>
-    <numFmt numFmtId="223" formatCode="#,##0.0_);[Red]\(#,##0.0\)"/>
-    <numFmt numFmtId="224" formatCode="0.0%_);[Red]\(0.0%\)"/>
-    <numFmt numFmtId="225" formatCode="0.00_);\(0.00\);0.00_)"/>
-    <numFmt numFmtId="226" formatCode="#,##0\x"/>
-    <numFmt numFmtId="227" formatCode="&quot;TKR&quot;\ 0"/>
-    <numFmt numFmtId="228" formatCode=".%\,\(0.%%;\t"/>
-    <numFmt numFmtId="229" formatCode="&quot;$&quot;#,###.0\ \ "/>
-    <numFmt numFmtId="230" formatCode="#,##0.00\x_);[Red]\(#,##0.00\x\)"/>
-    <numFmt numFmtId="231" formatCode="#,##0.000_);\(#,##0.000\)"/>
-    <numFmt numFmtId="232" formatCode="#,##0.00\x_);[Red]\(#,##0.00\x\);&quot;--  &quot;"/>
-    <numFmt numFmtId="233" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="234" formatCode="0.0\x_);[Red]\(0.0\x\)"/>
-    <numFmt numFmtId="235" formatCode="0.0\ "/>
-    <numFmt numFmtId="236" formatCode="&quot;$&quot;#,##0.0;\(&quot;$&quot;#,##0.00\)"/>
-    <numFmt numFmtId="237" formatCode="#,##0.00%_);\(#,##0.00%\)"/>
-    <numFmt numFmtId="238" formatCode="0.00\%;\-0.00\%;0.00\%"/>
-    <numFmt numFmtId="239" formatCode="0.0%\ ;\(0.0%\)"/>
-    <numFmt numFmtId="240" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="241" formatCode="&quot;$&quot;0.00\ "/>
-    <numFmt numFmtId="242" formatCode="0.0\ \ \ \ \ "/>
-    <numFmt numFmtId="243" formatCode="0.00\x;\-0.00\x;0.00\x"/>
-    <numFmt numFmtId="244" formatCode="&quot;$&quot;#,##0.000_);\(&quot;$&quot;#,##0.000\)"/>
-    <numFmt numFmtId="245" formatCode="#,##0.0_);\(#,##0.0\);_(* &quot;-&quot;_)"/>
-    <numFmt numFmtId="246" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="247" formatCode="0.00%_);[Red]\(0.00%\)"/>
-    <numFmt numFmtId="248" formatCode="#,##0.0\x_);\(#,##0.0\x\)"/>
-    <numFmt numFmtId="249" formatCode="#,##0.00\x_);\(#,##0.00\x\)"/>
-    <numFmt numFmtId="250" formatCode="###0&quot;E&quot;_)"/>
+    <numFmt numFmtId="192" formatCode="#,##0.00_);\(#,##0\)"/>
+    <numFmt numFmtId="193" formatCode="#,##0.0%_);\(#,##0.0%\)"/>
+    <numFmt numFmtId="194" formatCode="0.0\ \x"/>
+    <numFmt numFmtId="195" formatCode="#,##0.00\ ;\(#,##0.00\)"/>
+    <numFmt numFmtId="196" formatCode="&quot;$&quot;#,##0.00\ ;\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="197" formatCode="0.0%_);\(0.0%\)"/>
+    <numFmt numFmtId="198" formatCode="0.000\ \x&quot;rate&quot;"/>
+    <numFmt numFmtId="199" formatCode="#,##0.000_);[Red]\(#,##0.000\)"/>
+    <numFmt numFmtId="200" formatCode="0.00_);\(0.00\);0.00"/>
+    <numFmt numFmtId="201" formatCode="\C&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="202" formatCode="#,##0%_);\(#,##0.0%\)"/>
+    <numFmt numFmtId="203" formatCode="_(* #,##0.00000000_);_(* \(#,##0.00000000\);_(* &quot;-&quot;?_);_(@_)"/>
+    <numFmt numFmtId="204" formatCode="mmm\-d\-yyyy"/>
+    <numFmt numFmtId="205" formatCode="mmm\-yyyy"/>
+    <numFmt numFmtId="206" formatCode="yyyy"/>
+    <numFmt numFmtId="207" formatCode="0.00\x&quot;rate&quot;"/>
+    <numFmt numFmtId="208" formatCode="0.0&quot;  &quot;"/>
+    <numFmt numFmtId="209" formatCode="&quot;$&quot;#,##0.0\ ;[Red]\(&quot;$&quot;#,##0\)"/>
+    <numFmt numFmtId="210" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;?_);_(@_)"/>
+    <numFmt numFmtId="211" formatCode="&quot;$&quot;#,##0.000_);[Red]\(&quot;$&quot;#,##0.000\)"/>
+    <numFmt numFmtId="212" formatCode="&quot;$&quot;#,##0.00&quot;A&quot;;[Red]\(&quot;$&quot;#,##0.00\)&quot;A&quot;"/>
+    <numFmt numFmtId="213" formatCode="#,##0.0\ ;[Red]\(&quot;$&quot;#,##0\)"/>
+    <numFmt numFmtId="214" formatCode="&quot;$&quot;#,##0.00&quot;E&quot;;[Red]\(&quot;$&quot;#,##0.00\)&quot;E&quot;"/>
+    <numFmt numFmtId="215" formatCode="_([$€-2]* #,##0.00_);_([$€-2]* \(#,##0.00\);_([$€-2]* &quot;-&quot;??_)"/>
+    <numFmt numFmtId="216" formatCode="#,##0.00;\(#,##0.00\)"/>
+    <numFmt numFmtId="217" formatCode=".%\,\(0.0%%;\t"/>
+    <numFmt numFmtId="218" formatCode="#,##0.0_);[Red]\(#,##0.0\)"/>
+    <numFmt numFmtId="219" formatCode="0.0%_);[Red]\(0.0%\)"/>
+    <numFmt numFmtId="220" formatCode="0.00_);\(0.00\);0.00_)"/>
+    <numFmt numFmtId="221" formatCode="#,##0\x"/>
+    <numFmt numFmtId="222" formatCode="&quot;TKR&quot;\ 0"/>
+    <numFmt numFmtId="223" formatCode=".%\,\(0.%%;\t"/>
+    <numFmt numFmtId="224" formatCode="&quot;$&quot;#,###.0\ \ "/>
+    <numFmt numFmtId="225" formatCode="#,##0.00\x_);[Red]\(#,##0.00\x\)"/>
+    <numFmt numFmtId="226" formatCode="#,##0.000_);\(#,##0.000\)"/>
+    <numFmt numFmtId="227" formatCode="#,##0.00\x_);[Red]\(#,##0.00\x\);&quot;--  &quot;"/>
+    <numFmt numFmtId="228" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="229" formatCode="0.0\x_);[Red]\(0.0\x\)"/>
+    <numFmt numFmtId="230" formatCode="0.0\ "/>
+    <numFmt numFmtId="231" formatCode="&quot;$&quot;#,##0.0;\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="232" formatCode="#,##0.00%_);\(#,##0.00%\)"/>
+    <numFmt numFmtId="233" formatCode="0.00\%;\-0.00\%;0.00\%"/>
+    <numFmt numFmtId="234" formatCode="0.0%\ ;\(0.0%\)"/>
+    <numFmt numFmtId="235" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="236" formatCode="&quot;$&quot;0.00\ "/>
+    <numFmt numFmtId="237" formatCode="0.0\ \ \ \ \ "/>
+    <numFmt numFmtId="238" formatCode="0.00\x;\-0.00\x;0.00\x"/>
+    <numFmt numFmtId="239" formatCode="&quot;$&quot;#,##0.000_);\(&quot;$&quot;#,##0.000\)"/>
+    <numFmt numFmtId="240" formatCode="#,##0.0_);\(#,##0.0\);_(* &quot;-&quot;_)"/>
+    <numFmt numFmtId="241" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="242" formatCode="0.00%_);[Red]\(0.00%\)"/>
+    <numFmt numFmtId="243" formatCode="#,##0.0\x_);\(#,##0.0\x\)"/>
+    <numFmt numFmtId="244" formatCode="#,##0.00\x_);\(#,##0.00\x\)"/>
+    <numFmt numFmtId="245" formatCode="###0&quot;E&quot;_)"/>
+    <numFmt numFmtId="246" formatCode="0.0000"/>
+    <numFmt numFmtId="247" formatCode="0.000"/>
+    <numFmt numFmtId="248" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="118">
     <font>
@@ -1599,19 +1593,19 @@
   <cellStyleXfs count="187">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="38"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="38"/>
-    <xf numFmtId="197" fontId="8" fillId="0" borderId="38" applyAlignment="1">
+    <xf numFmtId="192" fontId="8" fillId="0" borderId="38" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="198" fontId="8" fillId="2" borderId="38"/>
-    <xf numFmtId="199" fontId="8" fillId="2" borderId="38"/>
-    <xf numFmtId="198" fontId="8" fillId="2" borderId="38"/>
-    <xf numFmtId="200" fontId="8" fillId="2" borderId="38"/>
-    <xf numFmtId="201" fontId="8" fillId="2" borderId="38" applyAlignment="1">
+    <xf numFmtId="193" fontId="8" fillId="2" borderId="38"/>
+    <xf numFmtId="194" fontId="8" fillId="2" borderId="38"/>
+    <xf numFmtId="193" fontId="8" fillId="2" borderId="38"/>
+    <xf numFmtId="195" fontId="8" fillId="2" borderId="38"/>
+    <xf numFmtId="196" fontId="8" fillId="2" borderId="38" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="202" fontId="9" fillId="0" borderId="38"/>
+    <xf numFmtId="197" fontId="9" fillId="0" borderId="38"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="38"/>
-    <xf numFmtId="203" fontId="11" fillId="0" borderId="38"/>
+    <xf numFmtId="198" fontId="11" fillId="0" borderId="38"/>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="38"/>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="38"/>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="38"/>
@@ -1638,7 +1632,7 @@
     <xf numFmtId="0" fontId="13" fillId="20" borderId="38"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="38"/>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="38"/>
-    <xf numFmtId="204" fontId="15" fillId="0" borderId="38"/>
+    <xf numFmtId="199" fontId="15" fillId="0" borderId="38"/>
     <xf numFmtId="38" fontId="15" fillId="0" borderId="38" applyProtection="1">
       <protection locked="0" hidden="0"/>
     </xf>
@@ -1647,10 +1641,10 @@
       <alignment horizontal="centerContinuous"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="21" borderId="5"/>
-    <xf numFmtId="204" fontId="15" fillId="0" borderId="38" applyProtection="1">
+    <xf numFmtId="199" fontId="15" fillId="0" borderId="38" applyProtection="1">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="204" fontId="15" fillId="0" borderId="6"/>
+    <xf numFmtId="199" fontId="15" fillId="0" borderId="6"/>
     <xf numFmtId="0" fontId="19" fillId="22" borderId="7"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="38" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -1668,35 +1662,35 @@
     <xf numFmtId="0" fontId="22" fillId="23" borderId="38" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="205" fontId="10" fillId="0" borderId="38" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="200" fontId="10" fillId="0" borderId="38" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="38"/>
     <xf numFmtId="7" fontId="24" fillId="0" borderId="38"/>
     <xf numFmtId="5" fontId="21" fillId="0" borderId="38"/>
-    <xf numFmtId="206" fontId="11" fillId="0" borderId="38" applyAlignment="1">
+    <xf numFmtId="201" fontId="11" fillId="0" borderId="38" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="207" fontId="8" fillId="2" borderId="9" applyAlignment="1">
+    <xf numFmtId="202" fontId="8" fillId="2" borderId="9" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="208" fontId="8" fillId="2" borderId="9" applyAlignment="1">
+    <xf numFmtId="203" fontId="8" fillId="2" borderId="9" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="207" fontId="8" fillId="2" borderId="9" applyAlignment="1">
+    <xf numFmtId="202" fontId="8" fillId="2" borderId="9" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="15" fontId="25" fillId="0" borderId="38"/>
-    <xf numFmtId="209" fontId="23" fillId="24" borderId="38"/>
-    <xf numFmtId="210" fontId="25" fillId="0" borderId="8"/>
+    <xf numFmtId="204" fontId="23" fillId="24" borderId="38"/>
+    <xf numFmtId="205" fontId="25" fillId="0" borderId="8"/>
     <xf numFmtId="14" fontId="26" fillId="0" borderId="38" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="211" fontId="26" fillId="0" borderId="38" applyAlignment="1">
+    <xf numFmtId="206" fontId="26" fillId="0" borderId="38" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="212" fontId="11" fillId="0" borderId="38"/>
+    <xf numFmtId="207" fontId="11" fillId="0" borderId="38"/>
     <xf numFmtId="8" fontId="15" fillId="0" borderId="38"/>
     <xf numFmtId="6" fontId="15" fillId="0" borderId="38" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1704,48 +1698,48 @@
     <xf numFmtId="6" fontId="15" fillId="0" borderId="38"/>
     <xf numFmtId="39" fontId="8" fillId="25" borderId="38"/>
     <xf numFmtId="7" fontId="8" fillId="25" borderId="38"/>
-    <xf numFmtId="213" fontId="8" fillId="25" borderId="38"/>
-    <xf numFmtId="214" fontId="8" fillId="0" borderId="38"/>
-    <xf numFmtId="215" fontId="8" fillId="25" borderId="38"/>
-    <xf numFmtId="216" fontId="8" fillId="25" borderId="38"/>
-    <xf numFmtId="217" fontId="16" fillId="0" borderId="38" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="208" fontId="8" fillId="25" borderId="38"/>
+    <xf numFmtId="209" fontId="8" fillId="0" borderId="38"/>
+    <xf numFmtId="210" fontId="8" fillId="25" borderId="38"/>
+    <xf numFmtId="211" fontId="8" fillId="25" borderId="38"/>
+    <xf numFmtId="212" fontId="16" fillId="0" borderId="38" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="218" fontId="8" fillId="0" borderId="38"/>
-    <xf numFmtId="219" fontId="16" fillId="0" borderId="38" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="213" fontId="8" fillId="0" borderId="38"/>
+    <xf numFmtId="214" fontId="16" fillId="0" borderId="38" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="220" fontId="10" fillId="0" borderId="38"/>
+    <xf numFmtId="215" fontId="10" fillId="0" borderId="38"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="38"/>
-    <xf numFmtId="202" fontId="8" fillId="0" borderId="10"/>
-    <xf numFmtId="221" fontId="8" fillId="2" borderId="9" applyAlignment="1">
+    <xf numFmtId="197" fontId="8" fillId="0" borderId="10"/>
+    <xf numFmtId="216" fontId="8" fillId="2" borderId="9" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="222" fontId="8" fillId="2" borderId="9" applyAlignment="1">
+    <xf numFmtId="217" fontId="8" fillId="2" borderId="9" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="221" fontId="8" fillId="2" borderId="9" applyAlignment="1">
+    <xf numFmtId="216" fontId="8" fillId="2" borderId="9" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="223" fontId="15" fillId="0" borderId="38" applyProtection="1">
+    <xf numFmtId="218" fontId="15" fillId="0" borderId="38" applyProtection="1">
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="5" borderId="38"/>
-    <xf numFmtId="224" fontId="29" fillId="0" borderId="38"/>
-    <xf numFmtId="202" fontId="30" fillId="0" borderId="38" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="219" fontId="29" fillId="0" borderId="38"/>
+    <xf numFmtId="197" fontId="30" fillId="0" borderId="38" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="223" fontId="11" fillId="26" borderId="11"/>
+    <xf numFmtId="218" fontId="11" fillId="26" borderId="11"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="12"/>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="13"/>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="14"/>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="38"/>
-    <xf numFmtId="223" fontId="34" fillId="0" borderId="38"/>
+    <xf numFmtId="218" fontId="34" fillId="0" borderId="38"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="38"/>
-    <xf numFmtId="204" fontId="15" fillId="0" borderId="38"/>
+    <xf numFmtId="199" fontId="15" fillId="0" borderId="38"/>
     <xf numFmtId="38" fontId="15" fillId="0" borderId="38" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0" hidden="0"/>
@@ -1759,7 +1753,7 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="17" fontId="37" fillId="27" borderId="38"/>
-    <xf numFmtId="225" fontId="10" fillId="0" borderId="38" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="220" fontId="10" fillId="0" borderId="38" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -1770,26 +1764,26 @@
     <xf numFmtId="173" fontId="15" fillId="0" borderId="38" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="226" fontId="8" fillId="0" borderId="38" applyAlignment="1">
+    <xf numFmtId="221" fontId="8" fillId="0" borderId="38" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="227" fontId="8" fillId="25" borderId="38" applyAlignment="1">
+    <xf numFmtId="222" fontId="8" fillId="25" borderId="38" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="228" fontId="8" fillId="0" borderId="38" applyAlignment="1">
+    <xf numFmtId="223" fontId="8" fillId="0" borderId="38" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="226" fontId="8" fillId="0" borderId="38" applyAlignment="1">
+    <xf numFmtId="221" fontId="8" fillId="0" borderId="38" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="202" fontId="40" fillId="0" borderId="38" applyAlignment="1">
+    <xf numFmtId="197" fontId="40" fillId="0" borderId="38" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="202" fontId="40" fillId="0" borderId="38"/>
-    <xf numFmtId="229" fontId="8" fillId="2" borderId="9" applyAlignment="1">
+    <xf numFmtId="197" fontId="40" fillId="0" borderId="38"/>
+    <xf numFmtId="224" fontId="8" fillId="2" borderId="9" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="230" fontId="15" fillId="0" borderId="38"/>
+    <xf numFmtId="225" fontId="15" fillId="0" borderId="38"/>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="38" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="1" hidden="1"/>
@@ -1798,62 +1792,62 @@
     <xf numFmtId="37" fontId="24" fillId="0" borderId="38"/>
     <xf numFmtId="175" fontId="10" fillId="0" borderId="38"/>
     <xf numFmtId="39" fontId="10" fillId="0" borderId="38"/>
-    <xf numFmtId="231" fontId="10" fillId="0" borderId="38"/>
+    <xf numFmtId="226" fontId="10" fillId="0" borderId="38"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="38"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="38"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="38"/>
-    <xf numFmtId="232" fontId="23" fillId="0" borderId="38"/>
+    <xf numFmtId="227" fontId="23" fillId="0" borderId="38"/>
     <xf numFmtId="0" fontId="12" fillId="29" borderId="17"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="38"/>
-    <xf numFmtId="233" fontId="10" fillId="0" borderId="38"/>
+    <xf numFmtId="228" fontId="10" fillId="0" borderId="38"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="38"/>
     <xf numFmtId="0" fontId="42" fillId="21" borderId="18"/>
-    <xf numFmtId="234" fontId="15" fillId="0" borderId="38" applyAlignment="1">
+    <xf numFmtId="229" fontId="15" fillId="0" borderId="38" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="0" borderId="38"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="38"/>
-    <xf numFmtId="235" fontId="8" fillId="25" borderId="38"/>
+    <xf numFmtId="230" fontId="8" fillId="25" borderId="38"/>
     <xf numFmtId="9" fontId="15" fillId="0" borderId="38" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="236" fontId="8" fillId="0" borderId="38"/>
+    <xf numFmtId="231" fontId="8" fillId="0" borderId="38"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="38"/>
-    <xf numFmtId="198" fontId="10" fillId="0" borderId="38"/>
-    <xf numFmtId="237" fontId="10" fillId="0" borderId="38"/>
+    <xf numFmtId="193" fontId="10" fillId="0" borderId="38"/>
+    <xf numFmtId="232" fontId="10" fillId="0" borderId="38"/>
+    <xf numFmtId="233" fontId="10" fillId="0" borderId="38" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="219" fontId="15" fillId="0" borderId="38"/>
+    <xf numFmtId="8" fontId="15" fillId="0" borderId="38"/>
+    <xf numFmtId="199" fontId="15" fillId="0" borderId="38" applyProtection="1">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="218" fontId="15" fillId="0" borderId="38"/>
+    <xf numFmtId="38" fontId="15" fillId="0" borderId="38"/>
+    <xf numFmtId="195" fontId="8" fillId="2" borderId="19" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="234" fontId="44" fillId="2" borderId="38"/>
+    <xf numFmtId="235" fontId="8" fillId="2" borderId="38"/>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="38" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="236" fontId="8" fillId="2" borderId="38" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="237" fontId="8" fillId="2" borderId="9" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="238" fontId="10" fillId="0" borderId="38" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="224" fontId="15" fillId="0" borderId="38"/>
-    <xf numFmtId="8" fontId="15" fillId="0" borderId="38"/>
-    <xf numFmtId="204" fontId="15" fillId="0" borderId="38" applyProtection="1">
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="223" fontId="15" fillId="0" borderId="38"/>
-    <xf numFmtId="38" fontId="15" fillId="0" borderId="38"/>
-    <xf numFmtId="200" fontId="8" fillId="2" borderId="19" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="239" fontId="44" fillId="2" borderId="38"/>
-    <xf numFmtId="240" fontId="8" fillId="2" borderId="38"/>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="38" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
-    </xf>
-    <xf numFmtId="241" fontId="8" fillId="2" borderId="38" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="242" fontId="8" fillId="2" borderId="9" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="243" fontId="10" fillId="0" borderId="38" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="223" fontId="26" fillId="0" borderId="38"/>
+    <xf numFmtId="218" fontId="26" fillId="0" borderId="38"/>
     <xf numFmtId="0" fontId="46" fillId="0" borderId="38" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -1861,10 +1855,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="1" hidden="1"/>
     </xf>
-    <xf numFmtId="204" fontId="15" fillId="0" borderId="38" applyProtection="1">
+    <xf numFmtId="199" fontId="15" fillId="0" borderId="38" applyProtection="1">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="244" fontId="26" fillId="0" borderId="38" applyAlignment="1">
+    <xf numFmtId="239" fontId="26" fillId="0" borderId="38" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="38" fontId="10" fillId="0" borderId="38"/>
@@ -1882,40 +1876,40 @@
     <xf numFmtId="0" fontId="52" fillId="0" borderId="38" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="245" fontId="53" fillId="0" borderId="38" applyAlignment="1">
+    <xf numFmtId="240" fontId="53" fillId="0" borderId="38" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="246" fontId="53" fillId="0" borderId="38" applyAlignment="1">
+    <xf numFmtId="241" fontId="53" fillId="0" borderId="38" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="23" fillId="0" borderId="38" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="216" fontId="54" fillId="0" borderId="38"/>
-    <xf numFmtId="247" fontId="55" fillId="0" borderId="38" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="211" fontId="54" fillId="0" borderId="38"/>
+    <xf numFmtId="242" fontId="55" fillId="0" borderId="38" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="247" fontId="55" fillId="0" borderId="38"/>
-    <xf numFmtId="247" fontId="56" fillId="0" borderId="38" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="242" fontId="55" fillId="0" borderId="38"/>
+    <xf numFmtId="242" fontId="56" fillId="0" borderId="38" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="247" fontId="56" fillId="0" borderId="38" applyProtection="1">
+    <xf numFmtId="242" fontId="56" fillId="0" borderId="38" applyProtection="1">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="223" fontId="15" fillId="0" borderId="38" applyProtection="1">
+    <xf numFmtId="218" fontId="15" fillId="0" borderId="38" applyProtection="1">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="223" fontId="54" fillId="0" borderId="38"/>
+    <xf numFmtId="218" fontId="54" fillId="0" borderId="38"/>
     <xf numFmtId="49" fontId="57" fillId="0" borderId="38"/>
-    <xf numFmtId="248" fontId="10" fillId="0" borderId="38"/>
-    <xf numFmtId="249" fontId="10" fillId="0" borderId="38"/>
+    <xf numFmtId="243" fontId="10" fillId="0" borderId="38"/>
+    <xf numFmtId="244" fontId="10" fillId="0" borderId="38"/>
     <xf numFmtId="0" fontId="58" fillId="0" borderId="38"/>
     <xf numFmtId="0" fontId="59" fillId="1" borderId="38" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="223" fontId="60" fillId="0" borderId="38"/>
+    <xf numFmtId="218" fontId="60" fillId="0" borderId="38"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="38"/>
     <xf numFmtId="38" fontId="61" fillId="0" borderId="38" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1924,10 +1918,10 @@
     <xf numFmtId="0" fontId="63" fillId="0" borderId="21"/>
     <xf numFmtId="0" fontId="64" fillId="0" borderId="38"/>
     <xf numFmtId="1" fontId="15" fillId="0" borderId="38"/>
-    <xf numFmtId="250" fontId="24" fillId="0" borderId="38"/>
-    <xf numFmtId="244" fontId="16" fillId="0" borderId="38"/>
+    <xf numFmtId="245" fontId="24" fillId="0" borderId="38"/>
+    <xf numFmtId="239" fontId="16" fillId="0" borderId="38"/>
   </cellStyleXfs>
-  <cellXfs count="470">
+  <cellXfs count="433">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2695,18 +2689,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="116" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="116" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="117" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="70" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="192" fontId="0" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="193" fontId="70" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="248" fontId="0" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="247" fontId="70" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="247" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="117" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="192" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="248" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="190" fontId="70" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="173" fontId="73" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="190" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -2716,7 +2711,7 @@
     <xf numFmtId="190" fontId="117" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="173" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="182" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="194" fontId="75" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="246" fontId="75" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="190" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2724,93 +2719,33 @@
     </xf>
     <xf numFmtId="190" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="173" fontId="5" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="195" fontId="0" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="196" fontId="66" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="182" fontId="0" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="66" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="66" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="190" fontId="70" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="190" fontId="65" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="193" fontId="70" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="193" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="247" fontId="70" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="247" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="173" fontId="70" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="5" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="5" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="117" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="173" fontId="5" fillId="32" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="173" fontId="4" fillId="32" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="173" fontId="4" fillId="32" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="195" fontId="4" fillId="32" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="195" fontId="5" fillId="32" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="195" fontId="4" fillId="32" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="173" fontId="5" fillId="32" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="173" fontId="4" fillId="32" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="173" fontId="4" fillId="32" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="195" fontId="4" fillId="32" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="190" fontId="4" fillId="32" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="190" fontId="4" fillId="32" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="190" fontId="5" fillId="32" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="190" fontId="4" fillId="32" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="194" fontId="7" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="246" fontId="7" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="246" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="73" fillId="44" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="193" fontId="5" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="193" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="247" fontId="5" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="117" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="193" fontId="117" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="117" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="182" fontId="5" fillId="44" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="44" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="182" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="182" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="182" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
+    <xf numFmtId="247" fontId="117" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="1" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="192" fontId="0" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="193" fontId="70" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="192" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="194" fontId="75" fillId="0" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="195" fontId="0" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="196" fontId="66" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="193" fontId="70" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="193" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="195" fontId="4" fillId="32" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="195" fontId="5" fillId="32" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="195" fontId="4" fillId="32" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="195" fontId="4" fillId="32" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="194" fontId="7" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="193" fontId="5" fillId="44" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="193" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="193" fontId="117" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="187">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3158,1875 +3093,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>ZoomInfo LBOMODEL2 — Base vs AI-SDR Strategy</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-      <overlay val="1"/>
-    </title>
-    <plotArea>
-      <layout/>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <varyColors val="1"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>Strategy_Summary!$C$49</f>
-              <strCache>
-                <ptCount val="1"/>
-                <pt idx="0">
-                  <v>Base</v>
-                </pt>
-              </strCache>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <invertIfNegative val="1"/>
-          <cat>
-            <strRef>
-              <f>Strategy_Summary!$B$50:$B$55</f>
-              <strCache>
-                <ptCount val="6"/>
-                <pt idx="0">
-                  <v>Y2 EBITDA margin %</v>
-                </pt>
-                <pt idx="1">
-                  <v>Y2 margin bps vs base</v>
-                </pt>
-                <pt idx="2">
-                  <v>Y5 EBITDA ($m)</v>
-                </pt>
-                <pt idx="3">
-                  <v>Exit equity ($m)</v>
-                </pt>
-                <pt idx="4">
-                  <v>MOIC (x)</v>
-                </pt>
-                <pt idx="5">
-                  <v>IRR (%)</v>
-                </pt>
-              </strCache>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>Strategy_Summary!$C$50:$C$55</f>
-              <numCache>
-                <formatCode>General</formatCode>
-                <ptCount val="6"/>
-                <pt idx="0">
-                  <v>10.85</v>
-                </pt>
-                <pt idx="1">
-                  <v>-422.75</v>
-                </pt>
-                <pt idx="2">
-                  <v>212.21</v>
-                </pt>
-                <pt idx="3">
-                  <v>2201.62</v>
-                </pt>
-                <pt idx="4">
-                  <v>1.18</v>
-                </pt>
-                <pt idx="5">
-                  <v>3.3</v>
-                </pt>
-              </numCache>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>Strategy_Summary!$D$49</f>
-              <strCache>
-                <ptCount val="1"/>
-                <pt idx="0">
-                  <v>AI-SDR</v>
-                </pt>
-              </strCache>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <invertIfNegative val="1"/>
-          <cat>
-            <strRef>
-              <f>Strategy_Summary!$B$50:$B$55</f>
-              <strCache>
-                <ptCount val="6"/>
-                <pt idx="0">
-                  <v>Y2 EBITDA margin %</v>
-                </pt>
-                <pt idx="1">
-                  <v>Y2 margin bps vs base</v>
-                </pt>
-                <pt idx="2">
-                  <v>Y5 EBITDA ($m)</v>
-                </pt>
-                <pt idx="3">
-                  <v>Exit equity ($m)</v>
-                </pt>
-                <pt idx="4">
-                  <v>MOIC (x)</v>
-                </pt>
-                <pt idx="5">
-                  <v>IRR (%)</v>
-                </pt>
-              </strCache>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>Strategy_Summary!$D$50:$D$55</f>
-              <numCache>
-                <formatCode>General</formatCode>
-                <ptCount val="6"/>
-                <pt idx="0">
-                  <v>18.83</v>
-                </pt>
-                <pt idx="1">
-                  <v>374.85</v>
-                </pt>
-                <pt idx="2">
-                  <v>477.4</v>
-                </pt>
-                <pt idx="3">
-                  <v>6206.15</v>
-                </pt>
-                <pt idx="4">
-                  <v>3.32</v>
-                </pt>
-                <pt idx="5">
-                  <v>27.1</v>
-                </pt>
-              </numCache>
-            </numRef>
-          </val>
-        </ser>
-        <dLbls>
-          <showLegendKey val="0"/>
-          <showVal val="0"/>
-          <showCatName val="0"/>
-          <showSerName val="0"/>
-          <showPercent val="0"/>
-          <showBubbleSize val="0"/>
-        </dLbls>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="1"/>
-        <axPos val="b"/>
-        <numFmt formatCode="General" sourceLinked="1"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <crossAx val="100"/>
-        <crosses val="autoZero"/>
-        <auto val="1"/>
-        <lblAlgn val="ctr"/>
-        <lblOffset val="100"/>
-        <noMultiLvlLbl val="1"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="1"/>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <numFmt formatCode="General" sourceLinked="1"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <crossAx val="10"/>
-        <crosses val="autoZero"/>
-        <crossBetween val="between"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-      <overlay val="1"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>Initial debt by tranche ($m)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-      <overlay val="1"/>
-    </title>
-    <plotArea>
-      <layout/>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <varyColors val="1"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>Debt_Sweep_AI!$G$11</f>
-              <strCache>
-                <ptCount val="1"/>
-                <pt idx="0">
-                  <v>Amount ($m)</v>
-                </pt>
-              </strCache>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <invertIfNegative val="1"/>
-          <dLbls>
-            <spPr>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-            <showLegendKey val="1"/>
-            <showVal val="1"/>
-            <showCatName val="1"/>
-            <showSerName val="1"/>
-            <showPercent val="1"/>
-            <showBubbleSize val="1"/>
-            <showLeaderLines val="0"/>
-          </dLbls>
-          <cat>
-            <strRef>
-              <f>Debt_Sweep_AI!$F$12:$F$14</f>
-              <strCache>
-                <ptCount val="3"/>
-                <pt idx="0">
-                  <v>Term Loan A principal</v>
-                </pt>
-                <pt idx="1">
-                  <v>Term Loan B principal</v>
-                </pt>
-                <pt idx="2">
-                  <v>Senior Notes principal</v>
-                </pt>
-              </strCache>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>Debt_Sweep_AI!$G$12:$G$14</f>
-              <numCache>
-                <formatCode>#,##0.00</formatCode>
-                <ptCount val="3"/>
-                <pt idx="0">
-                  <v>457.75</v>
-                </pt>
-                <pt idx="1">
-                  <v>274.65</v>
-                </pt>
-                <pt idx="2">
-                  <v>183.1</v>
-                </pt>
-              </numCache>
-            </numRef>
-          </val>
-        </ser>
-        <dLbls>
-          <showLegendKey val="1"/>
-          <showVal val="1"/>
-          <showCatName val="1"/>
-          <showSerName val="1"/>
-          <showPercent val="1"/>
-          <showBubbleSize val="1"/>
-        </dLbls>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="1"/>
-        <axPos val="b"/>
-        <numFmt formatCode="General" sourceLinked="1"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <crossAx val="100"/>
-        <crosses val="autoZero"/>
-        <auto val="1"/>
-        <lblAlgn val="ctr"/>
-        <lblOffset val="100"/>
-        <noMultiLvlLbl val="1"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="1"/>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-US"/>
-                  <a:t>$ millions</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-          <overlay val="1"/>
-        </title>
-        <numFmt formatCode="#,##0.00" sourceLinked="1"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <crossAx val="10"/>
-        <crosses val="autoZero"/>
-        <crossBetween val="between"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-      <overlay val="0"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1100"/>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US" sz="1100"/>
-              <a:t>DCF / LBO Football Field</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-      <layout>
-        <manualLayout>
-          <xMode val="edge"/>
-          <yMode val="edge"/>
-          <wMode val="factor"/>
-          <hMode val="factor"/>
-          <x val="0.3129162689269984"/>
-          <y val="0"/>
-        </manualLayout>
-      </layout>
-      <overlay val="0"/>
-    </title>
-    <plotArea>
-      <layout/>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="stacked"/>
-        <varyColors val="0"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>DCF!$C$114</f>
-              <strCache>
-                <ptCount val="1"/>
-                <pt idx="0">
-                  <v>Low</v>
-                </pt>
-              </strCache>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <invertIfNegative val="0"/>
-          <dLbls>
-            <spPr>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-            <dLblPos val="inEnd"/>
-            <showLegendKey val="0"/>
-            <showVal val="1"/>
-            <showCatName val="0"/>
-            <showSerName val="0"/>
-            <showPercent val="0"/>
-            <showBubbleSize val="0"/>
-            <showLeaderLines val="0"/>
-          </dLbls>
-          <cat>
-            <strRef>
-              <f>DCF!$B$115:$B$118</f>
-              <strCache>
-                <ptCount val="4"/>
-                <pt idx="0">
-                  <v>DCF Value at 6.3x-8.3x Exit EBITDA Range</v>
-                </pt>
-                <pt idx="1">
-                  <v>DCF Value at 2.0%-4.0% Perpetuity Range</v>
-                </pt>
-                <pt idx="2">
-                  <v>LBO Value at 15.0%-35.0% Sponsor Hurdle Rate</v>
-                </pt>
-                <pt idx="3">
-                  <v>52 Week Market High/Low</v>
-                </pt>
-              </strCache>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>DCF!$C$115:$C$118</f>
-              <numCache>
-                <formatCode>#,##0.0_);\(#,##0.0\);\-_);@_)</formatCode>
-                <ptCount val="4"/>
-                <pt idx="0">
-                  <v>20.64830251596892</v>
-                </pt>
-                <pt idx="1">
-                  <v>34.80938263855841</v>
-                </pt>
-                <pt idx="2">
-                  <v>45.45104265824024</v>
-                </pt>
-                <pt idx="3">
-                  <v>37.51</v>
-                </pt>
-              </numCache>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>DCF!$D$114</f>
-              <strCache>
-                <ptCount val="1"/>
-                <pt idx="0">
-                  <v>Diff.</v>
-                </pt>
-              </strCache>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <invertIfNegative val="0"/>
-          <cat>
-            <strRef>
-              <f>DCF!$B$115:$B$118</f>
-              <strCache>
-                <ptCount val="4"/>
-                <pt idx="0">
-                  <v>DCF Value at 6.3x-8.3x Exit EBITDA Range</v>
-                </pt>
-                <pt idx="1">
-                  <v>DCF Value at 2.0%-4.0% Perpetuity Range</v>
-                </pt>
-                <pt idx="2">
-                  <v>LBO Value at 15.0%-35.0% Sponsor Hurdle Rate</v>
-                </pt>
-                <pt idx="3">
-                  <v>52 Week Market High/Low</v>
-                </pt>
-              </strCache>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>DCF!$D$115:$D$118</f>
-              <numCache>
-                <formatCode>#,##0.0_);\(#,##0.0\);\-_);@_)</formatCode>
-                <ptCount val="4"/>
-                <pt idx="0">
-                  <v>11.06407079457684</v>
-                </pt>
-                <pt idx="1">
-                  <v>16.33763437516883</v>
-                </pt>
-                <pt idx="2">
-                  <v>13.0196839013479</v>
-                </pt>
-                <pt idx="3">
-                  <v>8.82</v>
-                </pt>
-              </numCache>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="2"/>
-          <order val="2"/>
-          <tx>
-            <strRef>
-              <f>DCF!$E$114</f>
-              <strCache>
-                <ptCount val="1"/>
-                <pt idx="0">
-                  <v>High</v>
-                </pt>
-              </strCache>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <invertIfNegative val="0"/>
-          <dLbls>
-            <spPr>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-            <dLblPos val="inBase"/>
-            <showLegendKey val="0"/>
-            <showVal val="1"/>
-            <showCatName val="0"/>
-            <showSerName val="0"/>
-            <showPercent val="0"/>
-            <showBubbleSize val="0"/>
-            <showLeaderLines val="0"/>
-          </dLbls>
-          <cat>
-            <strRef>
-              <f>DCF!$B$115:$B$118</f>
-              <strCache>
-                <ptCount val="4"/>
-                <pt idx="0">
-                  <v>DCF Value at 6.3x-8.3x Exit EBITDA Range</v>
-                </pt>
-                <pt idx="1">
-                  <v>DCF Value at 2.0%-4.0% Perpetuity Range</v>
-                </pt>
-                <pt idx="2">
-                  <v>LBO Value at 15.0%-35.0% Sponsor Hurdle Rate</v>
-                </pt>
-                <pt idx="3">
-                  <v>52 Week Market High/Low</v>
-                </pt>
-              </strCache>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>DCF!$E$115:$E$118</f>
-              <numCache>
-                <formatCode>#,##0.0_);\(#,##0.0\);\-_);@_)</formatCode>
-                <ptCount val="4"/>
-                <pt idx="0">
-                  <v>31.71237331054576</v>
-                </pt>
-                <pt idx="1">
-                  <v>51.14701701372724</v>
-                </pt>
-                <pt idx="2">
-                  <v>58.47072655958814</v>
-                </pt>
-                <pt idx="3">
-                  <v>46.33</v>
-                </pt>
-              </numCache>
-            </numRef>
-          </val>
-        </ser>
-        <dLbls>
-          <showLegendKey val="0"/>
-          <showVal val="0"/>
-          <showCatName val="0"/>
-          <showSerName val="0"/>
-          <showPercent val="0"/>
-          <showBubbleSize val="0"/>
-        </dLbls>
-        <gapWidth val="150"/>
-        <overlap val="100"/>
-        <axId val="388860856"/>
-        <axId val="388865952"/>
-      </barChart>
-      <catAx>
-        <axId val="388860856"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="b"/>
-        <numFmt formatCode="General" sourceLinked="0"/>
-        <majorTickMark val="out"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <crossAx val="388865952"/>
-        <crosses val="autoZero"/>
-        <auto val="1"/>
-        <lblAlgn val="ctr"/>
-        <lblOffset val="100"/>
-        <noMultiLvlLbl val="0"/>
-      </catAx>
-      <valAx>
-        <axId val="388865952"/>
-        <scaling>
-          <orientation val="minMax"/>
-          <max val="60"/>
-          <min val="10"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <numFmt formatCode="#,##0.0_);\(#,##0.0\);\-_);@_)" sourceLinked="1"/>
-        <majorTickMark val="out"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <crossAx val="388860856"/>
-        <crosses val="autoZero"/>
-        <crossBetween val="between"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-  <spPr>
-    <a:ln>
-      <a:noFill/>
-      <a:prstDash val="solid"/>
-    </a:ln>
-  </spPr>
-</chartSpace>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Wall Street Prep</author>
-  </authors>
-  <commentList>
-    <comment ref="H7" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Wall Street Prep:
-1 = Explicit EBITDA multiple assumption
-When a private company undergoes an LBO, the valuation discussion is expressed in terms of a multiple of EBITDA. Therefore, we input an EBITDA multiple assumption in this cell and work our way down to the implied offer value and offer value per share. 
-2 = Explicit offer price per share assumption
-However, offer value is sometimes also expressed in terms of offer price per share (usually when analyzing a public company), so rather that hardcoding an EBITDA multiple assumption, you could hard-code an offer price per share and work your way up to an implied EBITDA multiple. </t>
-      </text>
-    </comment>
-    <comment ref="D10" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-If the model "blows up" (i.e. REF and DIV/0 everywhere), turn the circuit breaker above on, and then immediately off again. 
-Why do we need this?
-This model has an intentional circularity in the calculation of interest expense and interest income. 
-Interest expense is calculated as interest rate times average current and prior period revolver debt balances. Since current period revolver balance is itself impacted by current period interest expense, the circularity exists.
-The same logic applies to interest expense.
-Setting Iterations in Excel
-Make sure that iterations are selected under Excel Options &gt; Formulas
-Removing circularity altogether
-To avoid a circularity altogether, calculate interest expense using prior period debt balances (as opposed to average balances).</t>
-      </text>
-    </comment>
-    <comment ref="B13" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Wall Street Prep:
-Input the last twelve months (LTM) EBITDA. </t>
-      </text>
-    </comment>
-    <comment ref="B14" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Include all debt and debt equivalents as of the most recent filing</t>
-      </text>
-    </comment>
-    <comment ref="B15" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Include all cash and equivalents as of most recent filing.</t>
-      </text>
-    </comment>
-    <comment ref="J26" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Accounting rules require that financing fees be capitalized and subsequently amortized over the term of the loan.
-This contrasts with the accounting treatment of transaction fees, which are expensed as incurred.</t>
-      </text>
-    </comment>
-    <comment ref="D27" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-$1.4 in excess cash used in BMC LBO</t>
-      </text>
-    </comment>
-    <comment ref="D28" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Up to $350m in availability on revolver with 5 year term</t>
-      </text>
-    </comment>
-    <comment ref="D29" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Originally $3.2b senior secured 7 year term loan reduced to $2.88b</t>
-      </text>
-    </comment>
-    <comment ref="D30" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Originally $1b second senior secured tranche, 7 year term loan reduced to 670m</t>
-      </text>
-    </comment>
-    <comment ref="D31" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Originally $1.38b high yield bond, matures 2021 increased to $1.625b.</t>
-      </text>
-    </comment>
-    <comment ref="C46" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Includes amortization expense</t>
-      </text>
-    </comment>
-    <comment ref="D46" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Includes amortization expense</t>
-      </text>
-    </comment>
-    <comment ref="E46" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Includes amortization expense</t>
-      </text>
-    </comment>
-    <comment ref="B47" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-includes capitalized financing fees, and D&amp;A from write-ups. Usually ignored by analysts when analyzing true ongoing profitability.</t>
-      </text>
-    </comment>
-    <comment ref="B59" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-includes capitalized financing fees, and D&amp;A from write-ups. Usually ignored by analysts when analyzing true ongoing profitability.</t>
-      </text>
-    </comment>
-    <comment ref="F61" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-BMC projections per Merger Proxy, p.72</t>
-      </text>
-    </comment>
-    <comment ref="G61" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-BMC projections per Merger Proxy, p.72</t>
-      </text>
-    </comment>
-    <comment ref="H61" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-BMC projections per Merger Proxy, p.72</t>
-      </text>
-    </comment>
-    <comment ref="I61" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-BMC projections per Merger Proxy, p.72</t>
-      </text>
-    </comment>
-    <comment ref="J61" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-BMC projections per Merger Proxy, p.72</t>
-      </text>
-    </comment>
-    <comment ref="F65" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-BMC projections per Merger Proxy, p.72</t>
-      </text>
-    </comment>
-    <comment ref="G65" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-BMC projections per Merger Proxy, p.72</t>
-      </text>
-    </comment>
-    <comment ref="H65" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-BMC projections per Merger Proxy, p.72</t>
-      </text>
-    </comment>
-    <comment ref="I65" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-BMC projections per Merger Proxy, p.72</t>
-      </text>
-    </comment>
-    <comment ref="J65" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-BMC projections per Merger Proxy, p.72</t>
-      </text>
-    </comment>
-    <comment ref="F70" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Tried to get close to BMC projections per Merger Proxy, p.72</t>
-      </text>
-    </comment>
-    <comment ref="D76" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Includes trade AR and both current &amp; non current finance receivables.</t>
-      </text>
-    </comment>
-    <comment ref="E76" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Includes trade AR and both current &amp; non current finance receivables.</t>
-      </text>
-    </comment>
-    <comment ref="D82" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Includes accrued expenses and both current and long term deferred revenue</t>
-      </text>
-    </comment>
-    <comment ref="E82" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Includes accrued expenses and both current and long term deferred revenue</t>
-      </text>
-    </comment>
-    <comment ref="F92" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Tried to approximate mangement guidance in Merger proxy p.72</t>
-      </text>
-    </comment>
-    <comment ref="G92" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Tried to approximate mangement guidance in Merger proxy p.72</t>
-      </text>
-    </comment>
-    <comment ref="H92" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Tried to approximate mangement guidance in Merger proxy p.72</t>
-      </text>
-    </comment>
-    <comment ref="I92" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Tried to approximate mangement guidance in Merger proxy p.72</t>
-      </text>
-    </comment>
-    <comment ref="J92" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Tried to approximate mangement guidance in Merger proxy p.72</t>
-      </text>
-    </comment>
-    <comment ref="C93" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Source: BMC 10K 2013 p. 72</t>
-      </text>
-    </comment>
-    <comment ref="D93" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Source: BMC 10K 2013 p. 72</t>
-      </text>
-    </comment>
-    <comment ref="E93" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Source: BMC 10K 2013 p. 72</t>
-      </text>
-    </comment>
-    <comment ref="K93" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Wall Street Prep:
-In an LBO where fixed asset purchases are limited to maintenance (as opposed to growth) capex, the ratio between capex and depreciation should converge to 1 over time, as new machines simply replace the absolesence of old machines.  </t>
-      </text>
-    </comment>
-    <comment ref="C98" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-BMC 2013 10K, CFS.</t>
-      </text>
-    </comment>
-    <comment ref="D98" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-BMC 2013 10K, CFS.</t>
-      </text>
-    </comment>
-    <comment ref="E98" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-BMC 2013 10K, CFS.</t>
-      </text>
-    </comment>
-    <comment ref="F98" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-BMC projections per Merger Proxy, p.72</t>
-      </text>
-    </comment>
-    <comment ref="G98" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-BMC projections per Merger Proxy, p.72</t>
-      </text>
-    </comment>
-    <comment ref="H98" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-BMC projections per Merger Proxy, p.72</t>
-      </text>
-    </comment>
-    <comment ref="I98" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-BMC projections per Merger Proxy, p.72</t>
-      </text>
-    </comment>
-    <comment ref="J98" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-BMC projections per Merger Proxy, p.72</t>
-      </text>
-    </comment>
-    <comment ref="C99" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Wall Street Prep:
-Source: BMC 2013 10K p. 60 </t>
-      </text>
-    </comment>
-    <comment ref="D99" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Wall Street Prep:
-Source: BMC 2013 10K p. 60 </t>
-      </text>
-    </comment>
-    <comment ref="E99" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Wall Street Prep:
-Source: BMC 2013 10K p. 60 </t>
-      </text>
-    </comment>
-    <comment ref="K99" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Wall Street Prep:
-In an LBO where fixed asset purchases are limited to maintenance (as opposed to growth) capex, the ratio between capex and depreciation should converge to 1 over time, as new machines simply replace the absolesence of old machines.  </t>
-      </text>
-    </comment>
-    <comment ref="F105" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-BMC projections per Merger Proxy, p.72</t>
-      </text>
-    </comment>
-    <comment ref="G105" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-BMC projections per Merger Proxy, p.72</t>
-      </text>
-    </comment>
-    <comment ref="H105" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-BMC projections per Merger Proxy, p.72</t>
-      </text>
-    </comment>
-    <comment ref="I105" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-BMC projections per Merger Proxy, p.72</t>
-      </text>
-    </comment>
-    <comment ref="J105" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-BMC projections per Merger Proxy, p.72</t>
-      </text>
-    </comment>
-    <comment ref="D107" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Wall Street Prep:
-Includes goodwill and other assets </t>
-      </text>
-    </comment>
-    <comment ref="E107" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Wall Street Prep:
-Includes goodwill and other assets </t>
-      </text>
-    </comment>
-    <comment ref="B117" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-includes capitalized financing fees, and D&amp;A from write-ups. Usually ignored by analysts when analyzing true ongoing profitability.</t>
-      </text>
-    </comment>
-    <comment ref="E166" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-% of available cash to be used.</t>
-      </text>
-    </comment>
-    <comment ref="E174" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-% of available cash to be used.</t>
-      </text>
-    </comment>
-    <comment ref="F198" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-For simplicity we will ignore the impact of financing fee amortization on the I/S and the corresponding addback on the CFS).</t>
-      </text>
-    </comment>
-    <comment ref="G198" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-For simplicity we will ignore the impact of financing fee amortization on the I/S and the corresponding addback on the CFS).</t>
-      </text>
-    </comment>
-    <comment ref="H198" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-For simplicity we will ignore the impact of financing fee amortization on the I/S and the corresponding addback on the CFS).</t>
-      </text>
-    </comment>
-    <comment ref="I198" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-For simplicity we will ignore the impact of financing fee amortization on the I/S and the corresponding addback on the CFS).</t>
-      </text>
-    </comment>
-    <comment ref="J198" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-For simplicity we will ignore the impact of financing fee amortization on the I/S and the corresponding addback on the CFS).</t>
-      </text>
-    </comment>
-    <comment ref="E232" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Wall Street Prep:
-In addition to dividends, preferred stock may also negotiate to receive warrants to increase their returns (aka "equity kicker"). This has the impact of diluting the sponsors and management equity at exit. </t>
-      </text>
-    </comment>
-    <comment ref="E233" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Wall Street Prep:
-In addition to interest, lenders (usually high yield subordinated notes) may also negotiate to receive warrants to increase their returns (aka "equity kicker"). This has the impact of diluting the sponsors and management equity at exit. </t>
-      </text>
-    </comment>
-    <comment ref="H267" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Fully diluted</t>
-      </text>
-    </comment>
-    <comment ref="E282" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Ignored effects of changes in model-derived offer value on transaction and financing fees for simplicity</t>
-      </text>
-    </comment>
-    <comment ref="F282" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Ignored effects of changes in model-derived offer value on transaction and financing fees for simplicity</t>
-      </text>
-    </comment>
-    <comment ref="G282" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Ignored effects of changes in model-derived offer value on transaction and financing fees for simplicity</t>
-      </text>
-    </comment>
-    <comment ref="H282" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Ignored effects of changes in model-derived offer value on transaction and financing fees for simplicity</t>
-      </text>
-    </comment>
-    <comment ref="I282" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Ignored effects of changes in model-derived offer value on transaction and financing fees for simplicity</t>
-      </text>
-    </comment>
-    <comment ref="J282" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Ignored effects of changes in model-derived offer value on transaction and financing fees for simplicity</t>
-      </text>
-    </comment>
-    <comment ref="G322" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Wall Street Prep:
-Management rollover is excluded from both sources &amp; uses because it is simultaneously a debit and credit to equity, creating a net impact of zero to equity. </t>
-      </text>
-    </comment>
-    <comment ref="H322" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Wall Street Prep:
-Management rollover is excluded from both sources &amp; uses because it is simultaneously a debit and credit to equity, creating a net impact of zero to equity. </t>
-      </text>
-    </comment>
-    <comment ref="B334" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Includes DTLs created in the LBO</t>
-      </text>
-    </comment>
-    <comment ref="I334" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-DTLs created in the LBO</t>
-      </text>
-    </comment>
-    <comment ref="B335" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Include legacy noncontrolling interests and preferred stock for simplicty</t>
-      </text>
-    </comment>
-    <comment ref="G339" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Excludes management rollover</t>
-      </text>
-    </comment>
-    <comment ref="F351" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Includes capitalized financing fees</t>
-      </text>
-    </comment>
-    <comment ref="G351" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Includes capitalized financing fees</t>
-      </text>
-    </comment>
-    <comment ref="H351" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Includes capitalized financing fees</t>
-      </text>
-    </comment>
-    <comment ref="I351" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Includes capitalized financing fees</t>
-      </text>
-    </comment>
-    <comment ref="J351" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Includes capitalized financing fees</t>
-      </text>
-    </comment>
-    <comment ref="K351" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Includes capitalized financing fees</t>
-      </text>
-    </comment>
-    <comment ref="F352" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Wall Street Prep:
-Includes goodwill created in the LBO </t>
-      </text>
-    </comment>
-    <comment ref="G352" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Wall Street Prep:
-Includes goodwill created in the LBO </t>
-      </text>
-    </comment>
-    <comment ref="H352" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Wall Street Prep:
-Includes goodwill created in the LBO </t>
-      </text>
-    </comment>
-    <comment ref="I352" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Wall Street Prep:
-Includes goodwill created in the LBO </t>
-      </text>
-    </comment>
-    <comment ref="J352" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Wall Street Prep:
-Includes goodwill created in the LBO </t>
-      </text>
-    </comment>
-    <comment ref="K352" authorId="0" shapeId="0">
-      <text>
-        <t xml:space="preserve">Wall Street Prep:
-Includes goodwill created in the LBO </t>
-      </text>
-    </comment>
-    <comment ref="F358" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Include all LBO created debt tranches</t>
-      </text>
-    </comment>
-    <comment ref="G358" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Include all LBO created debt tranches</t>
-      </text>
-    </comment>
-    <comment ref="H358" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Include all LBO created debt tranches</t>
-      </text>
-    </comment>
-    <comment ref="I358" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Include all LBO created debt tranches</t>
-      </text>
-    </comment>
-    <comment ref="J358" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Include all LBO created debt tranches</t>
-      </text>
-    </comment>
-    <comment ref="K358" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Include all LBO created debt tranches</t>
-      </text>
-    </comment>
-    <comment ref="G362" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-PF Equity, BOP
-+ NI, current period
--  Dividends common &amp; preferred, (PIK and cash)
-+ SBC, current period (debit to RE via NI needs to be offset by credit to Common stock)
--  Financing fee amortization (b/c we ignored its impact directly on the IS)
-PF Equity, EOP</t>
-      </text>
-    </comment>
-    <comment ref="H362" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-PF Equity, BOP
-+ NI, current period
--  Dividends common &amp; preferred, (PIK and cash)
-+ SBC, current period (debit to RE via NI needs to be offset by credit to Common stock)
--  Financing fee amortization (b/c we ignored its impact directly on the IS)
-PF Equity, EOP</t>
-      </text>
-    </comment>
-    <comment ref="I362" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-PF Equity, BOP
-+ NI, current period
--  Dividends common &amp; preferred, (PIK and cash)
-+ SBC, current period (debit to RE via NI needs to be offset by credit to Common stock)
--  Financing fee amortization (b/c we ignored its impact directly on the IS)
-PF Equity, EOP</t>
-      </text>
-    </comment>
-    <comment ref="J362" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-PF Equity, BOP
-+ NI, current period
--  Dividends common &amp; preferred, (PIK and cash)
-+ SBC, current period (debit to RE via NI needs to be offset by credit to Common stock)
--  Financing fee amortization (b/c we ignored its impact directly on the IS)
-PF Equity, EOP</t>
-      </text>
-    </comment>
-    <comment ref="K362" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-PF Equity, BOP
-+ NI, current period
--  Dividends common &amp; preferred, (PIK and cash)
-+ SBC, current period (debit to RE via NI needs to be offset by credit to Common stock)
--  Financing fee amortization (b/c we ignored its impact directly on the IS)
-PF Equity, EOP</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Wall Street Prep</author>
-  </authors>
-  <commentList>
-    <comment ref="C8" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Per AAPL Q2 10-Q, as of April 11, 2014</t>
-      </text>
-    </comment>
-    <comment ref="C36" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-By ignoring D&amp;A and Capex/Intangible Assets/SDC we are implicitly assuming that mature-company capital spending is just enough to offset the absolesence of older capital purchases.</t>
-      </text>
-    </comment>
-    <comment ref="J37" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Same as LBO exit multiple</t>
-      </text>
-    </comment>
-    <comment ref="C55" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Yield on 10 Year US Treasury</t>
-      </text>
-    </comment>
-    <comment ref="C56" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Derived from peers and relvered at BMC's new highly levered capital structure</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Wall Street Prep</author>
-  </authors>
-  <commentList>
-    <comment ref="E5" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-Hard-code to avoid circularity when offer price is derived from an explicit EBITDA multiple assumption.
-Deeper dive
-The circularity exists because for a given offer value, the more shares will lead to lower offer price per share, while the now lower offer price per share leads to fewer repurchases and a larger dilutive impact/share count, once again lowering the offer price per share and on and on...</t>
-      </text>
-    </comment>
-    <comment ref="C25" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-This tranche represents all unvested options - these typically vest upon a change of control.</t>
-      </text>
-    </comment>
-    <comment ref="D25" authorId="0" shapeId="0">
-      <text>
-        <t>Wall Street Prep:
-This tranche represents all unvested options - these typically vest upon a change of control.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>0</colOff>
-      <row>56</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="6480000" cy="3600000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>8</col>
-      <colOff>0</colOff>
-      <row>10</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="4320000" cy="2880000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>53578</colOff>
-      <row>93</row>
-      <rowOff>149424</rowOff>
-    </from>
-    <to>
-      <col>4</col>
-      <colOff>654844</colOff>
-      <row>112</row>
-      <rowOff>53578</rowOff>
-    </to>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook r:id="rId1">
-    <sheetNames>
-      <sheetName val="Historical Data"/>
-      <sheetName val="Forecast Drivers"/>
-      <sheetName val="Results"/>
-      <sheetName val="Valuation Summary"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1">
-        <row r="25">
-          <cell r="E25">
-            <v>0</v>
-          </cell>
-          <cell r="F25">
-            <v>0</v>
-          </cell>
-          <cell r="G25">
-            <v>0</v>
-          </cell>
-          <cell r="H25">
-            <v>0</v>
-          </cell>
-          <cell r="I25">
-            <v>0</v>
-          </cell>
-          <cell r="J25">
-            <v>0</v>
-          </cell>
-          <cell r="K25">
-            <v>0</v>
-          </cell>
-          <cell r="L25">
-            <v>0</v>
-          </cell>
-          <cell r="M25">
-            <v>0</v>
-          </cell>
-          <cell r="N25">
-            <v>0</v>
-          </cell>
-          <cell r="O25">
-            <v>0</v>
-          </cell>
-          <cell r="P25">
-            <v>0</v>
-          </cell>
-          <cell r="Q25">
-            <v>0</v>
-          </cell>
-          <cell r="R25">
-            <v>0</v>
-          </cell>
-          <cell r="S25">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="330">
-          <cell r="D330">
-            <v>1</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="2">
-        <row r="142">
-          <cell r="F142">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="145">
-          <cell r="F145">
-            <v>0</v>
-          </cell>
-          <cell r="G145">
-            <v>0</v>
-          </cell>
-          <cell r="H145">
-            <v>0</v>
-          </cell>
-          <cell r="I145">
-            <v>0</v>
-          </cell>
-          <cell r="J145">
-            <v>0</v>
-          </cell>
-          <cell r="K145">
-            <v>0</v>
-          </cell>
-          <cell r="L145">
-            <v>0</v>
-          </cell>
-          <cell r="M145">
-            <v>0</v>
-          </cell>
-          <cell r="N145">
-            <v>0</v>
-          </cell>
-          <cell r="O145">
-            <v>0</v>
-          </cell>
-          <cell r="P145">
-            <v>0</v>
-          </cell>
-          <cell r="Q145">
-            <v>0</v>
-          </cell>
-          <cell r="R145">
-            <v>0</v>
-          </cell>
-          <cell r="S145">
-            <v>0</v>
-          </cell>
-          <cell r="T145">
-            <v>0</v>
-          </cell>
-          <cell r="U145">
-            <v>0</v>
-          </cell>
-          <cell r="V145">
-            <v>0</v>
-          </cell>
-          <cell r="W145">
-            <v>0</v>
-          </cell>
-          <cell r="X145">
-            <v>0</v>
-          </cell>
-          <cell r="Y145">
-            <v>0</v>
-          </cell>
-          <cell r="Z145">
-            <v>0</v>
-          </cell>
-          <cell r="AA145">
-            <v>0</v>
-          </cell>
-          <cell r="AB145">
-            <v>0</v>
-          </cell>
-          <cell r="AC145">
-            <v>0</v>
-          </cell>
-          <cell r="AD145">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="182">
-          <cell r="E182">
-            <v>0</v>
-          </cell>
-          <cell r="F182">
-            <v>0</v>
-          </cell>
-          <cell r="G182">
-            <v>0</v>
-          </cell>
-          <cell r="H182">
-            <v>0</v>
-          </cell>
-          <cell r="I182">
-            <v>0</v>
-          </cell>
-          <cell r="J182">
-            <v>0</v>
-          </cell>
-          <cell r="K182">
-            <v>0</v>
-          </cell>
-          <cell r="L182">
-            <v>0</v>
-          </cell>
-          <cell r="M182">
-            <v>0</v>
-          </cell>
-          <cell r="N182">
-            <v>0</v>
-          </cell>
-          <cell r="O182">
-            <v>0</v>
-          </cell>
-          <cell r="P182">
-            <v>0</v>
-          </cell>
-          <cell r="Q182">
-            <v>0</v>
-          </cell>
-          <cell r="R182">
-            <v>0</v>
-          </cell>
-          <cell r="S182">
-            <v>0</v>
-          </cell>
-          <cell r="T182">
-            <v>0</v>
-          </cell>
-          <cell r="U182">
-            <v>0</v>
-          </cell>
-          <cell r="V182">
-            <v>0</v>
-          </cell>
-          <cell r="W182">
-            <v>0</v>
-          </cell>
-          <cell r="X182">
-            <v>0</v>
-          </cell>
-          <cell r="Y182">
-            <v>0</v>
-          </cell>
-          <cell r="Z182">
-            <v>0</v>
-          </cell>
-          <cell r="AA182">
-            <v>0</v>
-          </cell>
-          <cell r="AB182">
-            <v>0</v>
-          </cell>
-          <cell r="AC182">
-            <v>0</v>
-          </cell>
-          <cell r="AD182">
-            <v>0</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="3" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook r:id="rId1">
-    <sheetNames>
-      <sheetName val="Circ_ans"/>
-      <sheetName val="Circ"/>
-      <sheetName val="Reg 0"/>
-      <sheetName val="Reg_ans"/>
-      <sheetName val="CF"/>
-      <sheetName val="CF_ans"/>
-      <sheetName val="BoostToolkitClipBoard2010"/>
-      <sheetName val="DS0"/>
-      <sheetName val="DS0_ans"/>
-      <sheetName val="Data Set1"/>
-      <sheetName val="DataSet2"/>
-      <sheetName val="DataSet3"/>
-      <sheetName val="Other"/>
-      <sheetName val="DataSet4"/>
-      <sheetName val="Array0"/>
-      <sheetName val="Array1"/>
-      <sheetName val="Array2"/>
-      <sheetName val="Array3"/>
-      <sheetName val="Array4"/>
-      <sheetName val="Array5"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14">
-        <row r="5">
-          <cell r="B5" t="str">
-            <v>iPad</v>
-          </cell>
-          <cell r="C5">
-            <v>500</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="B6" t="str">
-            <v>iPod</v>
-          </cell>
-          <cell r="C6">
-            <v>200</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="B7" t="str">
-            <v>iPhone</v>
-          </cell>
-          <cell r="C7">
-            <v>400</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-      <sheetData sheetId="17"/>
-      <sheetData sheetId="18"/>
-      <sheetData sheetId="19"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -6717,7 +4783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E28"/>
+  <dimension ref="B2:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="1.7265625" customWidth="1" style="381" min="1" max="1"/>
@@ -6727,7 +4793,7 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" s="381" thickBot="1"/>
     <row r="2" ht="27" customHeight="1" s="381" thickBot="1">
-      <c r="B2" s="388" t="inlineStr">
+      <c r="B2" s="387" t="inlineStr">
         <is>
           <t>Diluted shares for ZoomInfo (GTM)</t>
         </is>
@@ -6752,10 +4818,18 @@
           <t>Offer price (LBO)</t>
         </is>
       </c>
-      <c r="E5" s="466">
+      <c r="E5" s="426">
         <f>LBO!H20</f>
         <v/>
       </c>
+      <c r="F5" s="427" t="n">
+        <v>5.0625</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>cached (formulas in E)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="B6" s="223" t="inlineStr">
@@ -6763,21 +4837,27 @@
           <t>Latest close (LBO)</t>
         </is>
       </c>
-      <c r="E6" s="442">
+      <c r="E6" s="428">
         <f>LBO!D8</f>
         <v/>
       </c>
+      <c r="F6" s="390" t="n">
+        <v>4.05</v>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="108" t="inlineStr">
         <is>
-          <t>Diluted shares outstanding (mm) — from LBO tab</t>
-        </is>
-      </c>
-      <c r="E7" s="467">
+          <t>Diluted shares outstanding (mm)</t>
+        </is>
+      </c>
+      <c r="E7" s="429">
         <f>LBO!H18</f>
         <v/>
       </c>
+      <c r="F7" s="393" t="n">
+        <v>307.294</v>
+      </c>
     </row>
     <row r="8">
       <c r="B8" s="26" t="inlineStr">
@@ -6785,9 +4865,8 @@
           <t>In-the-money exercisable options (mm)</t>
         </is>
       </c>
-      <c r="E8" s="461">
-        <f>E28</f>
-        <v/>
+      <c r="E8" s="416" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -6796,20 +4875,18 @@
           <t>Total proceeds ($mm)</t>
         </is>
       </c>
-      <c r="E9" s="404">
-        <f>SUMPRODUCT((D19:D27&lt;$E$5)*(C19:C27)*(D19:D27))</f>
-        <v/>
+      <c r="E9" s="405" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="26" t="inlineStr">
         <is>
-          <t>Total shares repurchased (mm) — treasury method</t>
-        </is>
-      </c>
-      <c r="E10" s="468">
-        <f>IF(E5=0,0,E9/E5)</f>
-        <v/>
+          <t>Total shares repurchased (mm)</t>
+        </is>
+      </c>
+      <c r="E10" s="393" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -6818,18 +4895,17 @@
           <t>Net dilutive options</t>
         </is>
       </c>
-      <c r="E11" s="468">
-        <f>E8-E10</f>
-        <v/>
+      <c r="E11" s="393" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="26" t="inlineStr">
         <is>
-          <t>Dilutive impact of shares from other securities</t>
-        </is>
-      </c>
-      <c r="E12" s="467" t="n">
+          <t>Dilutive impact of other securities</t>
+        </is>
+      </c>
+      <c r="E12" s="429" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6838,15 +4914,18 @@
       <c r="E13" s="105" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="445" t="inlineStr">
+      <c r="B14" s="430" t="inlineStr">
         <is>
           <t>Net diluted shares outstanding (mm)</t>
         </is>
       </c>
       <c r="D14" s="107" t="n"/>
-      <c r="E14" s="469">
+      <c r="E14" s="431">
         <f>E7+E11+E12</f>
         <v/>
+      </c>
+      <c r="F14" s="393" t="n">
+        <v>307.294</v>
       </c>
     </row>
     <row r="15">
@@ -6855,9 +4934,9 @@
       <c r="E15" s="38" t="n"/>
     </row>
     <row r="16">
-      <c r="B16" s="447" t="inlineStr">
-        <is>
-          <t>Options outstanding — GTM note</t>
+      <c r="B16" s="116" t="inlineStr">
+        <is>
+          <t>Options note</t>
         </is>
       </c>
       <c r="C16" s="13" t="n"/>
@@ -6867,7 +4946,7 @@
     <row r="17">
       <c r="B17" t="inlineStr">
         <is>
-          <t>LBO!H18 already stores diluted shares used for offer value / share. No ZoomInfo option-tranche lattice was provided in this workbook; leave option rows at 0 unless you add filing detail. Source map: Strategy_Summary!C17.</t>
+          <t>LBO!H18 stores diluted shares for offer value/share. No GTM option lattice — options left at 0.</t>
         </is>
       </c>
       <c r="C17" s="120" t="n"/>
@@ -6876,167 +4955,66 @@
     </row>
     <row r="18">
       <c r="B18" s="216" t="n"/>
-      <c r="C18" s="217" t="inlineStr">
-        <is>
-          <t>Out. shares</t>
-        </is>
-      </c>
-      <c r="D18" s="217" t="inlineStr">
-        <is>
-          <t>Exercise price</t>
-        </is>
-      </c>
-      <c r="E18" s="218" t="inlineStr">
-        <is>
-          <t>In-the-$-shares</t>
-        </is>
-      </c>
+      <c r="C18" s="217" t="n"/>
+      <c r="D18" s="217" t="n"/>
+      <c r="E18" s="218" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="216" t="n">
-        <v>1</v>
-      </c>
-      <c r="C19" s="448" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="449" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="450">
-        <f>IF(AND(C19&gt;0,D19&lt;$E$5),C19,0)</f>
-        <v/>
-      </c>
+      <c r="B19" s="216" t="n"/>
+      <c r="C19" s="217" t="n"/>
+      <c r="D19" s="217" t="n"/>
+      <c r="E19" s="218" t="n"/>
     </row>
     <row r="20">
-      <c r="B20" s="216" t="n">
-        <v>2</v>
-      </c>
-      <c r="C20" s="448" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" s="449" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="450">
-        <f>IF(AND(C20&gt;0,D20&lt;$E$5),C20,0)</f>
-        <v/>
-      </c>
+      <c r="B20" s="216" t="n"/>
+      <c r="C20" s="217" t="n"/>
+      <c r="D20" s="217" t="n"/>
+      <c r="E20" s="218" t="n"/>
     </row>
     <row r="21">
-      <c r="B21" s="216" t="n">
-        <v>3</v>
-      </c>
-      <c r="C21" s="448" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="449" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="450">
-        <f>IF(AND(C21&gt;0,D21&lt;$E$5),C21,0)</f>
-        <v/>
-      </c>
+      <c r="B21" s="216" t="n"/>
+      <c r="C21" s="217" t="n"/>
+      <c r="D21" s="217" t="n"/>
+      <c r="E21" s="218" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="216" t="n">
-        <v>4</v>
-      </c>
-      <c r="C22" s="448" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" s="449" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" s="450">
-        <f>IF(AND(C22&gt;0,D22&lt;$E$5),C22,0)</f>
-        <v/>
-      </c>
+      <c r="B22" s="216" t="n"/>
+      <c r="C22" s="217" t="n"/>
+      <c r="D22" s="217" t="n"/>
+      <c r="E22" s="218" t="n"/>
     </row>
     <row r="23">
-      <c r="B23" s="216" t="n">
-        <v>5</v>
-      </c>
-      <c r="C23" s="448" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="449" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="450">
-        <f>IF(AND(C23&gt;0,D23&lt;$E$5),C23,0)</f>
-        <v/>
-      </c>
+      <c r="B23" s="216" t="n"/>
+      <c r="C23" s="217" t="n"/>
+      <c r="D23" s="217" t="n"/>
+      <c r="E23" s="218" t="n"/>
     </row>
     <row r="24">
-      <c r="B24" s="216" t="n">
-        <v>6</v>
-      </c>
-      <c r="C24" s="448" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="449" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="450">
-        <f>IF(AND(C24&gt;0,D24&lt;$E$5),C24,0)</f>
-        <v/>
-      </c>
+      <c r="B24" s="216" t="n"/>
+      <c r="C24" s="217" t="n"/>
+      <c r="D24" s="217" t="n"/>
+      <c r="E24" s="218" t="n"/>
     </row>
     <row r="25">
-      <c r="B25" s="216" t="n">
-        <v>7</v>
-      </c>
-      <c r="C25" s="448" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" s="449" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="450">
-        <f>IF(AND(C25&gt;0,D25&lt;$E$5),C25,0)</f>
-        <v/>
-      </c>
+      <c r="B25" s="216" t="n"/>
+      <c r="C25" s="217" t="n"/>
+      <c r="D25" s="217" t="n"/>
+      <c r="E25" s="218" t="n"/>
     </row>
     <row r="26">
-      <c r="B26" s="216" t="n">
-        <v>8</v>
-      </c>
-      <c r="C26" s="448" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="449" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" s="450">
-        <f>IF(AND(C26&gt;0,D26&lt;$E$5),C26,0)</f>
-        <v/>
-      </c>
+      <c r="B26" s="216" t="n"/>
+      <c r="C26" s="217" t="n"/>
+      <c r="D26" s="217" t="n"/>
+      <c r="E26" s="218" t="n"/>
     </row>
     <row r="27">
-      <c r="B27" s="216" t="n">
-        <v>9</v>
-      </c>
-      <c r="C27" s="448" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="449" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="451">
-        <f>IF(AND(C27&gt;0,D27&lt;$E$5),C27,0)</f>
-        <v/>
-      </c>
+      <c r="B27" s="216" t="n"/>
+      <c r="C27" s="217" t="n"/>
+      <c r="D27" s="217" t="n"/>
+      <c r="E27" s="219" t="n"/>
     </row>
     <row r="28">
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>ITM options total</t>
-        </is>
-      </c>
-      <c r="E28" s="452">
-        <f>SUM(E19:E27)</f>
-        <v/>
-      </c>
+      <c r="E28" s="220" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7077,7 +5055,7 @@
           <t>52 week high</t>
         </is>
       </c>
-      <c r="E4" s="453" t="n">
+      <c r="E4" s="432" t="n">
         <v>12.51</v>
       </c>
     </row>
@@ -7087,14 +5065,14 @@
           <t>52 week low</t>
         </is>
       </c>
-      <c r="E5" s="453" t="n">
+      <c r="E5" s="432" t="n">
         <v>2.54</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Summary high/low from Yahoo Finance GTM 1y range (regularMarketPrice 4.05 matches LBO!D8). Daily OHLC rows below are legacy BMC template history and are not used by DCF.</t>
+          <t>GTM Yahoo 1y high/low. Legacy OHLC rows below are unused BMC history.</t>
         </is>
       </c>
     </row>
@@ -13007,7 +10985,6 @@
     <mergeCell ref="B3:F3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -13045,7 +11022,7 @@
     <row r="3">
       <c r="B3" t="inlineStr">
         <is>
-          <t>Each row states Where (Tab!Cell), the math location, commentary, and the formula meaning. Operating engine is LBO; DCF tab now consumes AI_Operating + Drivers + LBO + Debt_Sweep for GTM valuation.</t>
+          <t>Each row states Where (Tab!Cell), the math location, commentary, and the formula meaning. Not DCF-primary — LBO/operating engine.</t>
         </is>
       </c>
     </row>
@@ -14982,7 +12959,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -16092,7 +14068,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="2">
-      <c r="B2" s="386" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>vengeanceaiUSC-LBOMODEL4 — ZoomInfo (GTM) AI-SDR take-private</t>
         </is>
@@ -16117,7 +14093,7 @@
       <c r="M8" s="302" t="n"/>
     </row>
     <row r="11">
-      <c r="B11" s="387" t="inlineStr">
+      <c r="B11" s="386" t="inlineStr">
         <is>
           <t>Sample Modeling Template: The enclosed models are proprietary to Wall Street Prep and are designed for illustrative and training purposes only.  Distributing, sharing, duplicating or altering these models in any way is prohibited without the written consent of Wall Street Prep, Inc.  For more information about our training programs, please contact us at 800-646-3575 or visit us online at wallstreetprep.com.</t>
         </is>
@@ -16129,7 +14105,7 @@
     <row r="40">
       <c r="B40" t="inlineStr">
         <is>
-          <t>Open Strategy_Summary first — AI vs Base IRR; DCF/Shares now wired to GTM tabs</t>
+          <t>Open Strategy_Summary first — AI vs Base IRR and 500+ bps check</t>
         </is>
       </c>
     </row>
@@ -24735,7 +22711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:K118"/>
+  <dimension ref="B2:L118"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <cols>
     <col width="1.7265625" customWidth="1" style="381" min="1" max="1"/>
@@ -24750,7 +22726,7 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" s="381" thickBot="1"/>
     <row r="2" ht="27" customHeight="1" s="381" thickBot="1">
-      <c r="B2" s="388" t="inlineStr">
+      <c r="B2" s="387" t="inlineStr">
         <is>
           <t>Discounted Cash Flow Model for ZoomInfo (GTM)</t>
         </is>
@@ -24767,7 +22743,7 @@
     <row r="3">
       <c r="B3" s="51" t="inlineStr">
         <is>
-          <t>$ mm except per share — forecast from AI_Operating (AI-SDR thesis case)</t>
+          <t>$ mm except per share — AI_Operating thesis case</t>
         </is>
       </c>
     </row>
@@ -24775,7 +22751,7 @@
       <c r="B4" s="51" t="n"/>
     </row>
     <row r="5" ht="15.75" customHeight="1" s="381" thickBot="1">
-      <c r="B5" s="389" t="inlineStr">
+      <c r="B5" s="388" t="inlineStr">
         <is>
           <t>General assumptions</t>
         </is>
@@ -24788,10 +22764,18 @@
           <t>Share price as of last close</t>
         </is>
       </c>
-      <c r="C6" s="390">
+      <c r="C6" s="389">
         <f>LBO!D8</f>
         <v/>
       </c>
+      <c r="K6" s="390" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>cached</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="51" t="inlineStr">
@@ -24799,7 +22783,7 @@
           <t>Latest closing share price date</t>
         </is>
       </c>
-      <c r="C7" s="454">
+      <c r="C7" s="391">
         <f>LBO!D9</f>
         <v/>
       </c>
@@ -24810,9 +22794,12 @@
           <t>Diluted shares outstanding (mm)</t>
         </is>
       </c>
-      <c r="C8" s="455">
+      <c r="C8" s="392">
         <f>Shares!E14</f>
         <v/>
+      </c>
+      <c r="K8" s="393" t="n">
+        <v>307.294</v>
       </c>
     </row>
     <row r="9">
@@ -24825,10 +22812,13 @@
         <f>C59</f>
         <v/>
       </c>
+      <c r="K9" s="394" t="n">
+        <v>0.09290152684082101</v>
+      </c>
     </row>
     <row r="10"/>
     <row r="11" ht="15.75" customHeight="1" s="381" thickBot="1">
-      <c r="B11" s="393" t="inlineStr">
+      <c r="B11" s="395" t="inlineStr">
         <is>
           <t>Free cash flow buildup</t>
         </is>
@@ -24848,22 +22838,22 @@
           <t>Fiscal year</t>
         </is>
       </c>
-      <c r="C12" s="394" t="n">
+      <c r="C12" s="14" t="n">
         <v>2024</v>
       </c>
-      <c r="D12" s="394" t="n">
+      <c r="D12" s="14" t="n">
         <v>2025</v>
       </c>
-      <c r="E12" s="394" t="n">
+      <c r="E12" s="14" t="n">
         <v>2026</v>
       </c>
-      <c r="F12" s="394" t="n">
+      <c r="F12" s="15" t="n">
         <v>2027</v>
       </c>
-      <c r="G12" s="394" t="n">
+      <c r="G12" s="15" t="n">
         <v>2028</v>
       </c>
-      <c r="H12" s="394" t="n">
+      <c r="H12" s="15" t="n">
         <v>2029</v>
       </c>
       <c r="I12" s="15" t="n"/>
@@ -24875,22 +22865,22 @@
           <t>Fiscal year end date</t>
         </is>
       </c>
-      <c r="C13" s="456" t="n">
+      <c r="C13" s="396" t="n">
         <v>45657</v>
       </c>
-      <c r="D13" s="456" t="n">
+      <c r="D13" s="396" t="n">
         <v>46022</v>
       </c>
-      <c r="E13" s="456" t="n">
+      <c r="E13" s="396" t="n">
         <v>46387</v>
       </c>
-      <c r="F13" s="456" t="n">
+      <c r="F13" s="396" t="n">
         <v>46752</v>
       </c>
-      <c r="G13" s="456" t="n">
+      <c r="G13" s="396" t="n">
         <v>47118</v>
       </c>
-      <c r="H13" s="456" t="n">
+      <c r="H13" s="396" t="n">
         <v>47483</v>
       </c>
       <c r="I13" s="31" t="n"/>
@@ -24910,27 +22900,27 @@
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="C15" s="396">
+      <c r="C15" s="397">
         <f>AI_Operating!C13</f>
         <v/>
       </c>
-      <c r="D15" s="396">
+      <c r="D15" s="397">
         <f>AI_Operating!D13</f>
         <v/>
       </c>
-      <c r="E15" s="396">
+      <c r="E15" s="397">
         <f>AI_Operating!E13</f>
         <v/>
       </c>
-      <c r="F15" s="396">
+      <c r="F15" s="397">
         <f>AI_Operating!F13</f>
         <v/>
       </c>
-      <c r="G15" s="396">
+      <c r="G15" s="397">
         <f>AI_Operating!G13</f>
         <v/>
       </c>
-      <c r="H15" s="396">
+      <c r="H15" s="397">
         <f>AI_Operating!H13</f>
         <v/>
       </c>
@@ -24943,27 +22933,27 @@
           <t>EBIT</t>
         </is>
       </c>
-      <c r="C16" s="396">
+      <c r="C16" s="397">
         <f>AI_Operating!C16</f>
         <v/>
       </c>
-      <c r="D16" s="396">
+      <c r="D16" s="397">
         <f>AI_Operating!D16</f>
         <v/>
       </c>
-      <c r="E16" s="396">
+      <c r="E16" s="397">
         <f>AI_Operating!E16</f>
         <v/>
       </c>
-      <c r="F16" s="396">
+      <c r="F16" s="397">
         <f>AI_Operating!F16</f>
         <v/>
       </c>
-      <c r="G16" s="396">
+      <c r="G16" s="397">
         <f>AI_Operating!G16</f>
         <v/>
       </c>
-      <c r="H16" s="396">
+      <c r="H16" s="397">
         <f>AI_Operating!H16</f>
         <v/>
       </c>
@@ -24976,27 +22966,27 @@
           <t>Tax rate</t>
         </is>
       </c>
-      <c r="C17" s="397">
+      <c r="C17" s="398">
         <f>Assumptions_Drivers!$C$19</f>
         <v/>
       </c>
-      <c r="D17" s="397">
+      <c r="D17" s="398">
         <f>Assumptions_Drivers!$C$19</f>
         <v/>
       </c>
-      <c r="E17" s="397">
+      <c r="E17" s="398">
         <f>Assumptions_Drivers!$C$19</f>
         <v/>
       </c>
-      <c r="F17" s="397">
+      <c r="F17" s="398">
         <f>Assumptions_Drivers!$C$19</f>
         <v/>
       </c>
-      <c r="G17" s="397">
+      <c r="G17" s="398">
         <f>Assumptions_Drivers!$C$19</f>
         <v/>
       </c>
-      <c r="H17" s="397">
+      <c r="H17" s="398">
         <f>Assumptions_Drivers!$C$19</f>
         <v/>
       </c>
@@ -25009,27 +22999,27 @@
           <t>EBIAT (NOPAT)</t>
         </is>
       </c>
-      <c r="C18" s="398">
+      <c r="C18" s="399">
         <f>C16*(1-C17)</f>
         <v/>
       </c>
-      <c r="D18" s="398">
+      <c r="D18" s="399">
         <f>D16*(1-D17)</f>
         <v/>
       </c>
-      <c r="E18" s="398">
+      <c r="E18" s="399">
         <f>E16*(1-E17)</f>
         <v/>
       </c>
-      <c r="F18" s="398">
+      <c r="F18" s="399">
         <f>F16*(1-F17)</f>
         <v/>
       </c>
-      <c r="G18" s="398">
+      <c r="G18" s="399">
         <f>G16*(1-G17)</f>
         <v/>
       </c>
-      <c r="H18" s="398">
+      <c r="H18" s="399">
         <f>H16*(1-H17)</f>
         <v/>
       </c>
@@ -25045,23 +23035,23 @@
           <t>Depreciation and amortization</t>
         </is>
       </c>
-      <c r="D20" s="399">
+      <c r="D20" s="400">
         <f>AI_Operating!D15</f>
         <v/>
       </c>
-      <c r="E20" s="399">
+      <c r="E20" s="400">
         <f>AI_Operating!E15</f>
         <v/>
       </c>
-      <c r="F20" s="396">
+      <c r="F20" s="397">
         <f>AI_Operating!F15</f>
         <v/>
       </c>
-      <c r="G20" s="396">
+      <c r="G20" s="397">
         <f>AI_Operating!G15</f>
         <v/>
       </c>
-      <c r="H20" s="396">
+      <c r="H20" s="397">
         <f>AI_Operating!H15</f>
         <v/>
       </c>
@@ -25074,19 +23064,19 @@
           <t>Stock based compensation</t>
         </is>
       </c>
-      <c r="D21" s="399" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="399" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="396" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="396" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="396" t="n">
+      <c r="D21" s="400" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="400" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="397" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="397" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="397" t="n">
         <v>0</v>
       </c>
       <c r="I21" s="50" t="n"/>
@@ -25098,23 +23088,23 @@
           <t>Changes in net working capital</t>
         </is>
       </c>
-      <c r="D22" s="399">
+      <c r="D22" s="400">
         <f>AI_Operating!D20</f>
         <v/>
       </c>
-      <c r="E22" s="399">
+      <c r="E22" s="400">
         <f>AI_Operating!E20</f>
         <v/>
       </c>
-      <c r="F22" s="396">
+      <c r="F22" s="397">
         <f>AI_Operating!F20</f>
         <v/>
       </c>
-      <c r="G22" s="396">
+      <c r="G22" s="397">
         <f>AI_Operating!G20</f>
         <v/>
       </c>
-      <c r="H22" s="396">
+      <c r="H22" s="397">
         <f>AI_Operating!H20</f>
         <v/>
       </c>
@@ -25127,19 +23117,19 @@
           <t>Other assets &amp; liabilities</t>
         </is>
       </c>
-      <c r="D23" s="399" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="399" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="396" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="396" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="396" t="n">
+      <c r="D23" s="400" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="400" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="397" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="397" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="397" t="n">
         <v>0</v>
       </c>
       <c r="I23" s="50" t="n"/>
@@ -25151,23 +23141,23 @@
           <t>Unlevered CFO</t>
         </is>
       </c>
-      <c r="D24" s="399">
+      <c r="D24" s="400">
         <f>D18+D20+D21-D22+D23</f>
         <v/>
       </c>
-      <c r="E24" s="399">
+      <c r="E24" s="400">
         <f>E18+E20+E21-E22+E23</f>
         <v/>
       </c>
-      <c r="F24" s="400">
+      <c r="F24" s="401">
         <f>F18+F20+F21-F22+F23</f>
         <v/>
       </c>
-      <c r="G24" s="400">
+      <c r="G24" s="401">
         <f>G18+G20+G21-G22+G23</f>
         <v/>
       </c>
-      <c r="H24" s="400">
+      <c r="H24" s="401">
         <f>H18+H20+H21-H22+H23</f>
         <v/>
       </c>
@@ -25180,23 +23170,23 @@
           <t>Less: Capital expenditures</t>
         </is>
       </c>
-      <c r="D25" s="399">
+      <c r="D25" s="400">
         <f>-AI_Operating!D19</f>
         <v/>
       </c>
-      <c r="E25" s="399">
+      <c r="E25" s="400">
         <f>-AI_Operating!E19</f>
         <v/>
       </c>
-      <c r="F25" s="396">
+      <c r="F25" s="397">
         <f>-AI_Operating!F19</f>
         <v/>
       </c>
-      <c r="G25" s="396">
+      <c r="G25" s="397">
         <f>-AI_Operating!G19</f>
         <v/>
       </c>
-      <c r="H25" s="396">
+      <c r="H25" s="397">
         <f>-AI_Operating!H19</f>
         <v/>
       </c>
@@ -25209,47 +23199,47 @@
           <t>Less: Purchases of intangible assets</t>
         </is>
       </c>
-      <c r="D26" s="399" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" s="399" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" s="396" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" s="396" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="396" t="n">
+      <c r="D26" s="400" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="400" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="397" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="397" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="397" t="n">
         <v>0</v>
       </c>
       <c r="I26" s="50" t="n"/>
       <c r="J26" s="50" t="n"/>
     </row>
     <row r="27">
-      <c r="B27" s="401" t="inlineStr">
+      <c r="B27" s="402" t="inlineStr">
         <is>
           <t>Unlevered FCF</t>
         </is>
       </c>
-      <c r="D27" s="402">
+      <c r="D27" s="403">
         <f>D24+D25+D26</f>
         <v/>
       </c>
-      <c r="E27" s="402">
+      <c r="E27" s="403">
         <f>E24+E25+E26</f>
         <v/>
       </c>
-      <c r="F27" s="402">
+      <c r="F27" s="403">
         <f>F24+F25+F26</f>
         <v/>
       </c>
-      <c r="G27" s="402">
+      <c r="G27" s="403">
         <f>G24+G25+G26</f>
         <v/>
       </c>
-      <c r="H27" s="402">
+      <c r="H27" s="403">
         <f>H24+H25+H26</f>
         <v/>
       </c>
@@ -25262,19 +23252,19 @@
           <t>% growth</t>
         </is>
       </c>
-      <c r="E28" s="403">
+      <c r="E28" s="404">
         <f>IF(D27=0,0,E27/D27-1)</f>
         <v/>
       </c>
-      <c r="F28" s="403">
+      <c r="F28" s="404">
         <f>IF(E27=0,0,F27/E27-1)</f>
         <v/>
       </c>
-      <c r="G28" s="403">
+      <c r="G28" s="404">
         <f>IF(F27=0,0,G27/F27-1)</f>
         <v/>
       </c>
-      <c r="H28" s="403">
+      <c r="H28" s="404">
         <f>IF(G27=0,0,H27/G27-1)</f>
         <v/>
       </c>
@@ -25294,19 +23284,19 @@
           <t>Discount period (years, mid-year)</t>
         </is>
       </c>
-      <c r="D30" s="404" t="n">
+      <c r="D30" s="405" t="n">
         <v>0.5</v>
       </c>
-      <c r="E30" s="404" t="n">
+      <c r="E30" s="405" t="n">
         <v>1.5</v>
       </c>
-      <c r="F30" s="404" t="n">
+      <c r="F30" s="405" t="n">
         <v>2.5</v>
       </c>
-      <c r="G30" s="404" t="n">
+      <c r="G30" s="405" t="n">
         <v>3.5</v>
       </c>
-      <c r="H30" s="404" t="n">
+      <c r="H30" s="405" t="n">
         <v>4.5</v>
       </c>
       <c r="I30" s="48" t="n"/>
@@ -25334,7 +23324,7 @@
           <t>Midperiod adjustment factor</t>
         </is>
       </c>
-      <c r="C32" s="457">
+      <c r="C32" s="406">
         <f>(1+$C$9)^0.5</f>
         <v/>
       </c>
@@ -25345,23 +23335,23 @@
           <t>Present value of Unlevered FCF</t>
         </is>
       </c>
-      <c r="D33" s="399">
+      <c r="D33" s="400">
         <f>D27/(1+$C$9)^D30</f>
         <v/>
       </c>
-      <c r="E33" s="399">
+      <c r="E33" s="400">
         <f>E27/(1+$C$9)^E30</f>
         <v/>
       </c>
-      <c r="F33" s="406">
+      <c r="F33" s="407">
         <f>F27/(1+$C$9)^F30</f>
         <v/>
       </c>
-      <c r="G33" s="406">
+      <c r="G33" s="407">
         <f>G27/(1+$C$9)^G30</f>
         <v/>
       </c>
-      <c r="H33" s="406">
+      <c r="H33" s="407">
         <f>H27/(1+$C$9)^H30</f>
         <v/>
       </c>
@@ -25373,13 +23363,13 @@
       <c r="C34" s="6" t="n"/>
     </row>
     <row r="35" ht="15.75" customHeight="1" s="381" thickBot="1">
-      <c r="B35" s="389" t="inlineStr">
+      <c r="B35" s="388" t="inlineStr">
         <is>
           <t>Perpetuity approach</t>
         </is>
       </c>
       <c r="C35" s="44" t="n"/>
-      <c r="E35" s="389" t="inlineStr">
+      <c r="E35" s="388" t="inlineStr">
         <is>
           <t>Exit EBITDA multiple approach</t>
         </is>
@@ -25396,7 +23386,7 @@
           <t>Normalized FCFt+1</t>
         </is>
       </c>
-      <c r="C36" s="407">
+      <c r="C36" s="408">
         <f>H27*(1+C37)</f>
         <v/>
       </c>
@@ -25405,7 +23395,7 @@
           <t>Terminal year EBITDA</t>
         </is>
       </c>
-      <c r="H36" s="399">
+      <c r="H36" s="400">
         <f>H15</f>
         <v/>
       </c>
@@ -25417,7 +23407,7 @@
           <t>Long term growth rate (g)</t>
         </is>
       </c>
-      <c r="C37" s="408">
+      <c r="C37" s="409">
         <f>Assumptions_Drivers!C10</f>
         <v/>
       </c>
@@ -25426,7 +23416,7 @@
           <t>Terminal value EBITDA multiple</t>
         </is>
       </c>
-      <c r="H37" s="458">
+      <c r="H37" s="410">
         <f>Assumptions_Drivers!C20</f>
         <v/>
       </c>
@@ -25439,7 +23429,7 @@
           <t>Terminal value</t>
         </is>
       </c>
-      <c r="C38" s="399">
+      <c r="C38" s="400">
         <f>IF(($C$9-C37)&lt;=0,"NM",C36/($C$9-C37))</f>
         <v/>
       </c>
@@ -25448,7 +23438,7 @@
           <t>Terminal value</t>
         </is>
       </c>
-      <c r="H38" s="399">
+      <c r="H38" s="400">
         <f>H36*H37</f>
         <v/>
       </c>
@@ -25460,7 +23450,7 @@
           <t>Present value of terminal value</t>
         </is>
       </c>
-      <c r="C39" s="399">
+      <c r="C39" s="400">
         <f>IF(ISNUMBER(C38),C38/(1+$C$9)^H30,0)</f>
         <v/>
       </c>
@@ -25469,7 +23459,7 @@
           <t>Present value of terminal value</t>
         </is>
       </c>
-      <c r="H39" s="399">
+      <c r="H39" s="400">
         <f>H38/(1+$C$9)^H30</f>
         <v/>
       </c>
@@ -25481,7 +23471,7 @@
           <t>Present value of stage 1 cash flows</t>
         </is>
       </c>
-      <c r="C40" s="399">
+      <c r="C40" s="400">
         <f>SUM(D33:H33)</f>
         <v/>
       </c>
@@ -25490,32 +23480,35 @@
           <t>Present value of stage 1 cash flows</t>
         </is>
       </c>
-      <c r="H40" s="399">
+      <c r="H40" s="400">
         <f>C40</f>
         <v/>
       </c>
       <c r="J40" s="23" t="n"/>
     </row>
     <row r="41">
-      <c r="B41" s="401" t="inlineStr">
+      <c r="B41" s="402" t="inlineStr">
         <is>
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="C41" s="402">
+      <c r="C41" s="403">
         <f>C39+C40</f>
         <v/>
       </c>
-      <c r="E41" s="401" t="inlineStr">
+      <c r="E41" s="402" t="inlineStr">
         <is>
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="H41" s="402">
+      <c r="H41" s="403">
         <f>H39+H40</f>
         <v/>
       </c>
       <c r="J41" s="42" t="n"/>
+      <c r="K41" s="400" t="n">
+        <v>3641.734669903512</v>
+      </c>
     </row>
     <row r="42">
       <c r="B42" s="19" t="inlineStr">
@@ -25523,7 +23516,7 @@
           <t>Implied TV exit EBITDA multiple</t>
         </is>
       </c>
-      <c r="C42" s="459">
+      <c r="C42" s="411">
         <f>IF(H15=0,0,C38/H15)</f>
         <v/>
       </c>
@@ -25534,7 +23527,7 @@
       </c>
       <c r="F42" s="19" t="n"/>
       <c r="G42" s="19" t="n"/>
-      <c r="H42" s="411">
+      <c r="H42" s="412">
         <f>IF(H38=0,0,($C$9*H38-H27)/(H38+H27))</f>
         <v/>
       </c>
@@ -25546,13 +23539,13 @@
       <c r="J43" s="6" t="n"/>
     </row>
     <row r="44" ht="15.75" customHeight="1" s="381" thickBot="1">
-      <c r="B44" s="389" t="inlineStr">
+      <c r="B44" s="388" t="inlineStr">
         <is>
           <t>Net Debt</t>
         </is>
       </c>
       <c r="C44" s="44" t="n"/>
-      <c r="E44" s="389" t="inlineStr">
+      <c r="E44" s="388" t="inlineStr">
         <is>
           <t>Fair value per share</t>
         </is>
@@ -25569,7 +23562,7 @@
           <t>Cash &amp; equivalents (LBO latest)</t>
         </is>
       </c>
-      <c r="C45" s="412">
+      <c r="C45" s="413">
         <f>LBO!D15</f>
         <v/>
       </c>
@@ -25595,7 +23588,7 @@
           <t>Gross debt (LBO latest filing)</t>
         </is>
       </c>
-      <c r="C46" s="412">
+      <c r="C46" s="413">
         <f>ABS(LBO!D14)</f>
         <v/>
       </c>
@@ -25604,15 +23597,15 @@
           <t>Enterprise value</t>
         </is>
       </c>
-      <c r="H46" s="399">
+      <c r="H46" s="400">
         <f>H48+C47</f>
         <v/>
       </c>
-      <c r="I46" s="399">
+      <c r="I46" s="400">
         <f>C41</f>
         <v/>
       </c>
-      <c r="J46" s="399">
+      <c r="J46" s="400">
         <f>H41</f>
         <v/>
       </c>
@@ -25623,7 +23616,7 @@
           <t>Net debt</t>
         </is>
       </c>
-      <c r="C47" s="398">
+      <c r="C47" s="399">
         <f>C46-C45</f>
         <v/>
       </c>
@@ -25632,15 +23625,15 @@
           <t>Less: Net debt</t>
         </is>
       </c>
-      <c r="H47" s="399">
+      <c r="H47" s="400">
         <f>-C47</f>
         <v/>
       </c>
-      <c r="I47" s="399">
+      <c r="I47" s="400">
         <f>-C47</f>
         <v/>
       </c>
-      <c r="J47" s="399">
+      <c r="J47" s="400">
         <f>-C47</f>
         <v/>
       </c>
@@ -25654,21 +23647,21 @@
       </c>
       <c r="F48" s="22" t="n"/>
       <c r="G48" s="22" t="n"/>
-      <c r="H48" s="413">
+      <c r="H48" s="414">
         <f>LBO!H20*$C$8</f>
         <v/>
       </c>
-      <c r="I48" s="400">
+      <c r="I48" s="401">
         <f>I46+I47</f>
         <v/>
       </c>
-      <c r="J48" s="400">
+      <c r="J48" s="401">
         <f>J46+J47</f>
         <v/>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1" s="381" thickBot="1">
-      <c r="B49" s="389" t="inlineStr">
+      <c r="B49" s="388" t="inlineStr">
         <is>
           <t>Cost of capital assumptions</t>
         </is>
@@ -25679,15 +23672,15 @@
           <t>Diluted shares</t>
         </is>
       </c>
-      <c r="H49" s="460">
+      <c r="H49" s="415">
         <f>$C$8</f>
         <v/>
       </c>
-      <c r="I49" s="461">
+      <c r="I49" s="416">
         <f>$C$8</f>
         <v/>
       </c>
-      <c r="J49" s="461">
+      <c r="J49" s="416">
         <f>$C$8</f>
         <v/>
       </c>
@@ -25698,7 +23691,7 @@
           <t>Cost of debt (wtd TLA/TLB/Notes)</t>
         </is>
       </c>
-      <c r="C50" s="416">
+      <c r="C50" s="417">
         <f>(Debt_Sweep_AI!G12*Assumptions_Drivers!C27+Debt_Sweep_AI!G13*Assumptions_Drivers!C28+Debt_Sweep_AI!G14*(Assumptions_Drivers!C14+0.035))/Debt_Sweep_AI!G15</f>
         <v/>
       </c>
@@ -25707,18 +23700,26 @@
           <t>Equity value per share</t>
         </is>
       </c>
-      <c r="H50" s="417">
+      <c r="H50" s="418">
         <f>LBO!H20</f>
         <v/>
       </c>
-      <c r="I50" s="417">
+      <c r="I50" s="418">
         <f>IF(I49=0,0,I48/I49)</f>
         <v/>
       </c>
-      <c r="J50" s="417">
+      <c r="J50" s="418">
         <f>IF(J49=0,0,J48/J49)</f>
         <v/>
       </c>
+      <c r="K50" s="390" t="n">
+        <v>8.10863430429332</v>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>cached exit $/sh</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="B51" t="inlineStr">
@@ -25726,7 +23727,7 @@
           <t>Tax rate</t>
         </is>
       </c>
-      <c r="C51" s="403">
+      <c r="C51" s="404">
         <f>Assumptions_Drivers!C19</f>
         <v/>
       </c>
@@ -25740,11 +23741,11 @@
           <t>NM</t>
         </is>
       </c>
-      <c r="I51" s="403">
+      <c r="I51" s="404">
         <f>IF(H50=0,0,I50/H50-1)</f>
         <v/>
       </c>
-      <c r="J51" s="403">
+      <c r="J51" s="404">
         <f>IF(H50=0,0,J50/H50-1)</f>
         <v/>
       </c>
@@ -25755,7 +23756,7 @@
           <t>Debt (new LBO stack $m)</t>
         </is>
       </c>
-      <c r="C52" s="399">
+      <c r="C52" s="400">
         <f>Debt_Sweep_AI!G15</f>
         <v/>
       </c>
@@ -25766,7 +23767,7 @@
           <t>Debt as a % of total capital</t>
         </is>
       </c>
-      <c r="C53" s="418">
+      <c r="C53" s="419">
         <f>C52/(C52+C54)</f>
         <v/>
       </c>
@@ -25777,7 +23778,7 @@
           <t>Sponsor equity check ($m)</t>
         </is>
       </c>
-      <c r="C54" s="399">
+      <c r="C54" s="400">
         <f>Strategy_Summary!C20</f>
         <v/>
       </c>
@@ -25788,7 +23789,7 @@
           <t>Risk free rate (SOFR from Drivers)</t>
         </is>
       </c>
-      <c r="C55" s="419">
+      <c r="C55" s="420">
         <f>Assumptions_Drivers!C14</f>
         <v/>
       </c>
@@ -25799,7 +23800,7 @@
           <t>Beta (MODEL CONST — SaaS mid)</t>
         </is>
       </c>
-      <c r="C56" s="420" t="n">
+      <c r="C56" s="421" t="n">
         <v>1.25</v>
       </c>
     </row>
@@ -25809,7 +23810,7 @@
           <t>Market risk premium</t>
         </is>
       </c>
-      <c r="C57" s="408" t="n">
+      <c r="C57" s="409" t="n">
         <v>0.05</v>
       </c>
     </row>
@@ -25819,29 +23820,25 @@
           <t>Equity as % of total capital structure</t>
         </is>
       </c>
-      <c r="C58" s="403">
+      <c r="C58" s="404">
         <f>1-C53</f>
         <v/>
       </c>
     </row>
     <row r="59">
-      <c r="B59" s="401" t="inlineStr">
+      <c r="B59" s="402" t="inlineStr">
         <is>
           <t>Cost of capital (WACC)</t>
         </is>
       </c>
-      <c r="C59" s="421">
+      <c r="C59" s="422">
         <f>C58*(C55+C56*C57)+C53*C50*(1-C51)</f>
         <v/>
       </c>
     </row>
     <row r="60"/>
     <row r="61" ht="15.75" customHeight="1" s="381" thickBot="1">
-      <c r="B61" s="389" t="inlineStr">
-        <is>
-          <t>Sensitivity analysis</t>
-        </is>
-      </c>
+      <c r="B61" s="46" t="n"/>
       <c r="C61" s="44" t="n"/>
       <c r="D61" s="44" t="n"/>
       <c r="E61" s="44" t="n"/>
@@ -25854,11 +23851,7 @@
     </row>
     <row r="63" ht="17.25" customHeight="1" s="381">
       <c r="B63" s="22" t="n"/>
-      <c r="C63" s="83" t="inlineStr">
-        <is>
-          <t>Equity value per share (perpetuity)</t>
-        </is>
-      </c>
+      <c r="C63" s="83" t="n"/>
       <c r="D63" s="83" t="n"/>
       <c r="E63" s="83" t="n"/>
       <c r="F63" s="83" t="n"/>
@@ -25867,11 +23860,7 @@
     </row>
     <row r="64">
       <c r="C64" s="34" t="n"/>
-      <c r="D64" s="45" t="inlineStr">
-        <is>
-          <t>Long term growth rate (g):</t>
-        </is>
-      </c>
+      <c r="D64" s="45" t="n"/>
       <c r="E64" s="45" t="n"/>
       <c r="F64" s="45" t="n"/>
       <c r="G64" s="45" t="n"/>
@@ -25879,180 +23868,61 @@
     </row>
     <row r="65">
       <c r="B65" s="75" t="n"/>
-      <c r="C65" s="422">
-        <f>I50</f>
-        <v/>
-      </c>
-      <c r="D65" s="84" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="E65" s="85" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="F65" s="86" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="G65" s="85" t="n">
-        <v>0.025</v>
-      </c>
-      <c r="H65" s="87" t="n">
-        <v>0.03</v>
-      </c>
+      <c r="C65" s="82" t="n"/>
+      <c r="D65" s="84" t="n"/>
+      <c r="E65" s="85" t="n"/>
+      <c r="F65" s="86" t="n"/>
+      <c r="G65" s="85" t="n"/>
+      <c r="H65" s="87" t="n"/>
     </row>
     <row r="66">
-      <c r="C66" s="423" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="D66" s="424">
-        <f>IF(($C66-D$65)&lt;=0,"NM",(($C$40+($H$27*(1+D$65))/($C66-D$65))/(1+$C66)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="E66" s="424">
-        <f>IF(($C66-E$65)&lt;=0,"NM",(($C$40+($H$27*(1+E$65))/($C66-E$65))/(1+$C66)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="F66" s="424">
-        <f>IF(($C66-F$65)&lt;=0,"NM",(($C$40+($H$27*(1+F$65))/($C66-F$65))/(1+$C66)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="G66" s="424">
-        <f>IF(($C66-G$65)&lt;=0,"NM",(($C$40+($H$27*(1+G$65))/($C66-G$65))/(1+$C66)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="H66" s="424">
-        <f>IF(($C66-H$65)&lt;=0,"NM",(($C$40+($H$27*(1+H$65))/($C66-H$65))/(1+$C66)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
+      <c r="C66" s="88" t="n"/>
+      <c r="D66" s="63" t="n"/>
+      <c r="E66" s="63" t="n"/>
+      <c r="F66" s="63" t="n"/>
+      <c r="G66" s="63" t="n"/>
+      <c r="H66" s="63" t="n"/>
     </row>
     <row r="67">
-      <c r="C67" s="425" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D67" s="424">
-        <f>IF(($C67-D$65)&lt;=0,"NM",(($C$40+($H$27*(1+D$65))/($C67-D$65))/(1+$C67)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="E67" s="424">
-        <f>IF(($C67-E$65)&lt;=0,"NM",(($C$40+($H$27*(1+E$65))/($C67-E$65))/(1+$C67)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="F67" s="424">
-        <f>IF(($C67-F$65)&lt;=0,"NM",(($C$40+($H$27*(1+F$65))/($C67-F$65))/(1+$C67)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="G67" s="424">
-        <f>IF(($C67-G$65)&lt;=0,"NM",(($C$40+($H$27*(1+G$65))/($C67-G$65))/(1+$C67)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="H67" s="424">
-        <f>IF(($C67-H$65)&lt;=0,"NM",(($C$40+($H$27*(1+H$65))/($C67-H$65))/(1+$C67)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
+      <c r="C67" s="89" t="n"/>
+      <c r="D67" s="63" t="n"/>
+      <c r="E67" s="63" t="n"/>
+      <c r="F67" s="63" t="n"/>
+      <c r="G67" s="63" t="n"/>
+      <c r="H67" s="63" t="n"/>
     </row>
     <row r="68">
-      <c r="B68" s="75" t="inlineStr">
-        <is>
-          <t>WACC:</t>
-        </is>
-      </c>
-      <c r="C68" s="425" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="D68" s="424">
-        <f>IF(($C68-D$65)&lt;=0,"NM",(($C$40+($H$27*(1+D$65))/($C68-D$65))/(1+$C68)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="E68" s="424">
-        <f>IF(($C68-E$65)&lt;=0,"NM",(($C$40+($H$27*(1+E$65))/($C68-E$65))/(1+$C68)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="F68" s="424">
-        <f>IF(($C68-F$65)&lt;=0,"NM",(($C$40+($H$27*(1+F$65))/($C68-F$65))/(1+$C68)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="G68" s="424">
-        <f>IF(($C68-G$65)&lt;=0,"NM",(($C$40+($H$27*(1+G$65))/($C68-G$65))/(1+$C68)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="H68" s="424">
-        <f>IF(($C68-H$65)&lt;=0,"NM",(($C$40+($H$27*(1+H$65))/($C68-H$65))/(1+$C68)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
+      <c r="B68" s="75" t="n"/>
+      <c r="C68" s="89" t="n"/>
+      <c r="D68" s="63" t="n"/>
+      <c r="E68" s="63" t="n"/>
+      <c r="F68" s="63" t="n"/>
+      <c r="G68" s="63" t="n"/>
+      <c r="H68" s="63" t="n"/>
     </row>
     <row r="69">
-      <c r="C69" s="425" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="D69" s="424">
-        <f>IF(($C69-D$65)&lt;=0,"NM",(($C$40+($H$27*(1+D$65))/($C69-D$65))/(1+$C69)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="E69" s="424">
-        <f>IF(($C69-E$65)&lt;=0,"NM",(($C$40+($H$27*(1+E$65))/($C69-E$65))/(1+$C69)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="F69" s="424">
-        <f>IF(($C69-F$65)&lt;=0,"NM",(($C$40+($H$27*(1+F$65))/($C69-F$65))/(1+$C69)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="G69" s="424">
-        <f>IF(($C69-G$65)&lt;=0,"NM",(($C$40+($H$27*(1+G$65))/($C69-G$65))/(1+$C69)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="H69" s="424">
-        <f>IF(($C69-H$65)&lt;=0,"NM",(($C$40+($H$27*(1+H$65))/($C69-H$65))/(1+$C69)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
+      <c r="C69" s="89" t="n"/>
+      <c r="D69" s="63" t="n"/>
+      <c r="E69" s="63" t="n"/>
+      <c r="F69" s="63" t="n"/>
+      <c r="G69" s="63" t="n"/>
+      <c r="H69" s="63" t="n"/>
     </row>
     <row r="70">
-      <c r="C70" s="425" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="D70" s="424">
-        <f>IF(($C70-D$65)&lt;=0,"NM",(($C$40+($H$27*(1+D$65))/($C70-D$65))/(1+$C70)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="E70" s="424">
-        <f>IF(($C70-E$65)&lt;=0,"NM",(($C$40+($H$27*(1+E$65))/($C70-E$65))/(1+$C70)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="F70" s="424">
-        <f>IF(($C70-F$65)&lt;=0,"NM",(($C$40+($H$27*(1+F$65))/($C70-F$65))/(1+$C70)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="G70" s="424">
-        <f>IF(($C70-G$65)&lt;=0,"NM",(($C$40+($H$27*(1+G$65))/($C70-G$65))/(1+$C70)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="H70" s="424">
-        <f>IF(($C70-H$65)&lt;=0,"NM",(($C$40+($H$27*(1+H$65))/($C70-H$65))/(1+$C70)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
+      <c r="C70" s="89" t="n"/>
+      <c r="D70" s="63" t="n"/>
+      <c r="E70" s="63" t="n"/>
+      <c r="F70" s="63" t="n"/>
+      <c r="G70" s="63" t="n"/>
+      <c r="H70" s="63" t="n"/>
     </row>
     <row r="71">
-      <c r="C71" s="426" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="D71" s="424">
-        <f>IF(($C71-D$65)&lt;=0,"NM",(($C$40+($H$27*(1+D$65))/($C71-D$65))/(1+$C71)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="E71" s="424">
-        <f>IF(($C71-E$65)&lt;=0,"NM",(($C$40+($H$27*(1+E$65))/($C71-E$65))/(1+$C71)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="F71" s="424">
-        <f>IF(($C71-F$65)&lt;=0,"NM",(($C$40+($H$27*(1+F$65))/($C71-F$65))/(1+$C71)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="G71" s="424">
-        <f>IF(($C71-G$65)&lt;=0,"NM",(($C$40+($H$27*(1+G$65))/($C71-G$65))/(1+$C71)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
-      <c r="H71" s="424">
-        <f>IF(($C71-H$65)&lt;=0,"NM",(($C$40+($H$27*(1+H$65))/($C71-H$65))/(1+$C71)^$H$30-$C$47)/$C$8)</f>
-        <v/>
-      </c>
+      <c r="C71" s="90" t="n"/>
+      <c r="D71" s="63" t="n"/>
+      <c r="E71" s="63" t="n"/>
+      <c r="F71" s="63" t="n"/>
+      <c r="G71" s="63" t="n"/>
+      <c r="H71" s="63" t="n"/>
     </row>
     <row r="72">
       <c r="D72" s="63" t="n"/>
@@ -26062,11 +23932,7 @@
       <c r="H72" s="63" t="n"/>
     </row>
     <row r="73" ht="17.25" customHeight="1" s="381">
-      <c r="C73" s="83" t="inlineStr">
-        <is>
-          <t>Equity value per share (exit multiple)</t>
-        </is>
-      </c>
+      <c r="C73" s="83" t="n"/>
       <c r="D73" s="83" t="n"/>
       <c r="E73" s="83" t="n"/>
       <c r="F73" s="83" t="n"/>
@@ -26074,199 +23940,72 @@
       <c r="H73" s="83" t="n"/>
     </row>
     <row r="74">
-      <c r="D74" s="45" t="inlineStr">
-        <is>
-          <t>Exit EBITDA Multiple</t>
-        </is>
-      </c>
+      <c r="D74" s="45" t="n"/>
       <c r="E74" s="45" t="n"/>
       <c r="F74" s="45" t="n"/>
       <c r="G74" s="45" t="n"/>
       <c r="H74" s="45" t="n"/>
     </row>
     <row r="75">
-      <c r="C75" s="427">
-        <f>J50</f>
-        <v/>
-      </c>
-      <c r="D75" s="462" t="n">
-        <v>10.9</v>
-      </c>
-      <c r="E75" s="462" t="n">
-        <v>11.9</v>
-      </c>
-      <c r="F75" s="463" t="n">
-        <v>12.9</v>
-      </c>
-      <c r="G75" s="462" t="n">
-        <v>13.9</v>
-      </c>
-      <c r="H75" s="464" t="n">
-        <v>14.9</v>
-      </c>
+      <c r="C75" s="69" t="n"/>
+      <c r="D75" s="91" t="n"/>
+      <c r="E75" s="91" t="n"/>
+      <c r="F75" s="92" t="n"/>
+      <c r="G75" s="91" t="n"/>
+      <c r="H75" s="93" t="n"/>
     </row>
     <row r="76">
-      <c r="C76" s="431" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="D76" s="424">
-        <f>(($C$40+($H$15*D$75)/(1+$C76)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="E76" s="424">
-        <f>(($C$40+($H$15*E$75)/(1+$C76)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="F76" s="424">
-        <f>(($C$40+($H$15*F$75)/(1+$C76)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="G76" s="424">
-        <f>(($C$40+($H$15*G$75)/(1+$C76)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="H76" s="424">
-        <f>(($C$40+($H$15*H$75)/(1+$C76)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
+      <c r="C76" s="94" t="n"/>
+      <c r="D76" s="63" t="n"/>
+      <c r="E76" s="63" t="n"/>
+      <c r="F76" s="63" t="n"/>
+      <c r="G76" s="63" t="n"/>
+      <c r="H76" s="63" t="n"/>
     </row>
     <row r="77">
-      <c r="C77" s="432" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D77" s="424">
-        <f>(($C$40+($H$15*D$75)/(1+$C77)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="E77" s="424">
-        <f>(($C$40+($H$15*E$75)/(1+$C77)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="F77" s="424">
-        <f>(($C$40+($H$15*F$75)/(1+$C77)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="G77" s="424">
-        <f>(($C$40+($H$15*G$75)/(1+$C77)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="H77" s="424">
-        <f>(($C$40+($H$15*H$75)/(1+$C77)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
+      <c r="C77" s="95" t="n"/>
+      <c r="D77" s="63" t="n"/>
+      <c r="E77" s="63" t="n"/>
+      <c r="F77" s="63" t="n"/>
+      <c r="G77" s="63" t="n"/>
+      <c r="H77" s="63" t="n"/>
     </row>
     <row r="78">
-      <c r="B78" s="75" t="inlineStr">
-        <is>
-          <t>WACC:</t>
-        </is>
-      </c>
-      <c r="C78" s="432" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="D78" s="424">
-        <f>(($C$40+($H$15*D$75)/(1+$C78)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="E78" s="424">
-        <f>(($C$40+($H$15*E$75)/(1+$C78)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="F78" s="424">
-        <f>(($C$40+($H$15*F$75)/(1+$C78)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="G78" s="424">
-        <f>(($C$40+($H$15*G$75)/(1+$C78)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="H78" s="424">
-        <f>(($C$40+($H$15*H$75)/(1+$C78)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
+      <c r="B78" s="75" t="n"/>
+      <c r="C78" s="95" t="n"/>
+      <c r="D78" s="63" t="n"/>
+      <c r="E78" s="63" t="n"/>
+      <c r="F78" s="63" t="n"/>
+      <c r="G78" s="63" t="n"/>
+      <c r="H78" s="63" t="n"/>
     </row>
     <row r="79">
-      <c r="C79" s="432" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="D79" s="424">
-        <f>(($C$40+($H$15*D$75)/(1+$C79)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="E79" s="424">
-        <f>(($C$40+($H$15*E$75)/(1+$C79)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="F79" s="424">
-        <f>(($C$40+($H$15*F$75)/(1+$C79)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="G79" s="424">
-        <f>(($C$40+($H$15*G$75)/(1+$C79)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="H79" s="424">
-        <f>(($C$40+($H$15*H$75)/(1+$C79)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
+      <c r="C79" s="95" t="n"/>
+      <c r="D79" s="63" t="n"/>
+      <c r="E79" s="63" t="n"/>
+      <c r="F79" s="63" t="n"/>
+      <c r="G79" s="63" t="n"/>
+      <c r="H79" s="63" t="n"/>
     </row>
     <row r="80">
-      <c r="C80" s="432" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="D80" s="424">
-        <f>(($C$40+($H$15*D$75)/(1+$C80)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="E80" s="424">
-        <f>(($C$40+($H$15*E$75)/(1+$C80)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="F80" s="424">
-        <f>(($C$40+($H$15*F$75)/(1+$C80)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="G80" s="424">
-        <f>(($C$40+($H$15*G$75)/(1+$C80)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="H80" s="424">
-        <f>(($C$40+($H$15*H$75)/(1+$C80)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
+      <c r="C80" s="95" t="n"/>
+      <c r="D80" s="63" t="n"/>
+      <c r="E80" s="63" t="n"/>
+      <c r="F80" s="63" t="n"/>
+      <c r="G80" s="63" t="n"/>
+      <c r="H80" s="63" t="n"/>
     </row>
     <row r="81">
-      <c r="C81" s="433" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="D81" s="424">
-        <f>(($C$40+($H$15*D$75)/(1+$C81)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="E81" s="424">
-        <f>(($C$40+($H$15*E$75)/(1+$C81)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="F81" s="424">
-        <f>(($C$40+($H$15*F$75)/(1+$C81)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="G81" s="424">
-        <f>(($C$40+($H$15*G$75)/(1+$C81)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="H81" s="424">
-        <f>(($C$40+($H$15*H$75)/(1+$C81)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
+      <c r="C81" s="96" t="n"/>
+      <c r="D81" s="63" t="n"/>
+      <c r="E81" s="63" t="n"/>
+      <c r="F81" s="63" t="n"/>
+      <c r="G81" s="63" t="n"/>
+      <c r="H81" s="63" t="n"/>
     </row>
     <row r="82"/>
     <row r="83" ht="17.25" customHeight="1" s="381">
-      <c r="C83" s="83" t="inlineStr">
-        <is>
-          <t>Equity value per share</t>
-        </is>
-      </c>
+      <c r="C83" s="83" t="n"/>
       <c r="D83" s="83" t="n"/>
       <c r="E83" s="83" t="n"/>
       <c r="F83" s="83" t="n"/>
@@ -26274,206 +24013,99 @@
       <c r="H83" s="83" t="n"/>
     </row>
     <row r="84">
-      <c r="D84" s="45" t="inlineStr">
-        <is>
-          <t>Exit EBITDA Multiple</t>
-        </is>
-      </c>
+      <c r="D84" s="45" t="n"/>
       <c r="E84" s="45" t="n"/>
       <c r="F84" s="45" t="n"/>
       <c r="G84" s="45" t="n"/>
       <c r="H84" s="45" t="n"/>
     </row>
     <row r="85">
-      <c r="C85" s="102" t="inlineStr">
-        <is>
-          <t>EBITDA % of plan</t>
-        </is>
-      </c>
-      <c r="D85" s="424">
-        <f>J50</f>
-        <v/>
-      </c>
-      <c r="E85" s="465" t="n">
-        <v>10.9</v>
-      </c>
-      <c r="F85" s="462" t="n">
-        <v>11.9</v>
-      </c>
-      <c r="G85" s="463" t="n">
-        <v>12.9</v>
-      </c>
-      <c r="H85" s="464" t="n">
-        <v>13.9</v>
-      </c>
+      <c r="C85" s="102" t="n"/>
+      <c r="D85" s="72" t="n"/>
+      <c r="E85" s="97" t="n"/>
+      <c r="F85" s="91" t="n"/>
+      <c r="G85" s="92" t="n"/>
+      <c r="H85" s="93" t="n"/>
     </row>
     <row r="86">
-      <c r="C86" s="103" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="D86" s="435">
-        <f>$H$15*C86</f>
-        <v/>
-      </c>
-      <c r="E86" s="424">
-        <f>(($C$40+(D86*E$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="F86" s="424">
-        <f>(($C$40+(D86*F$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="G86" s="424">
-        <f>(($C$40+(D86*G$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="H86" s="424">
-        <f>(($C$40+(D86*H$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
+      <c r="C86" s="103" t="n"/>
+      <c r="D86" s="98" t="n"/>
+      <c r="E86" s="63" t="n"/>
+      <c r="F86" s="63" t="n"/>
+      <c r="G86" s="63" t="n"/>
+      <c r="H86" s="63" t="n"/>
     </row>
     <row r="87">
-      <c r="C87" s="104" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="D87" s="436">
-        <f>$H$15*C87</f>
-        <v/>
-      </c>
-      <c r="E87" s="424">
-        <f>(($C$40+(D87*E$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="F87" s="424">
-        <f>(($C$40+(D87*F$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="G87" s="424">
-        <f>(($C$40+(D87*G$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="H87" s="424">
-        <f>(($C$40+(D87*H$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
+      <c r="C87" s="104" t="n"/>
+      <c r="D87" s="99" t="n"/>
+      <c r="E87" s="63" t="n"/>
+      <c r="F87" s="63" t="n"/>
+      <c r="G87" s="63" t="n"/>
+      <c r="H87" s="63" t="n"/>
     </row>
     <row r="88">
-      <c r="C88" s="104" t="n">
-        <v>1</v>
-      </c>
-      <c r="D88" s="437">
-        <f>$H$15*C88</f>
-        <v/>
-      </c>
-      <c r="E88" s="424">
-        <f>(($C$40+(D88*E$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="F88" s="424">
-        <f>(($C$40+(D88*F$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="G88" s="424">
-        <f>(($C$40+(D88*G$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="H88" s="424">
-        <f>(($C$40+(D88*H$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
+      <c r="C88" s="104" t="n"/>
+      <c r="D88" s="100" t="n"/>
+      <c r="E88" s="63" t="n"/>
+      <c r="F88" s="63" t="n"/>
+      <c r="G88" s="63" t="n"/>
+      <c r="H88" s="63" t="n"/>
     </row>
     <row r="89">
-      <c r="C89" s="104" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="D89" s="436">
-        <f>$H$15*C89</f>
-        <v/>
-      </c>
-      <c r="E89" s="424">
-        <f>(($C$40+(D89*E$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="F89" s="424">
-        <f>(($C$40+(D89*F$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="G89" s="424">
-        <f>(($C$40+(D89*G$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="H89" s="424">
-        <f>(($C$40+(D89*H$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
+      <c r="C89" s="104" t="n"/>
+      <c r="D89" s="99" t="n"/>
+      <c r="E89" s="63" t="n"/>
+      <c r="F89" s="63" t="n"/>
+      <c r="G89" s="63" t="n"/>
+      <c r="H89" s="63" t="n"/>
     </row>
     <row r="90">
-      <c r="C90" s="104" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="D90" s="436">
-        <f>$H$15*C90</f>
-        <v/>
-      </c>
-      <c r="E90" s="424">
-        <f>(($C$40+(D90*E$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="F90" s="424">
-        <f>(($C$40+(D90*F$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="G90" s="424">
-        <f>(($C$40+(D90*G$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="H90" s="424">
-        <f>(($C$40+(D90*H$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
+      <c r="C90" s="104" t="n"/>
+      <c r="D90" s="99" t="n"/>
+      <c r="E90" s="63" t="n"/>
+      <c r="F90" s="63" t="n"/>
+      <c r="G90" s="63" t="n"/>
+      <c r="H90" s="63" t="n"/>
     </row>
     <row r="91">
-      <c r="C91" s="104" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="D91" s="438">
-        <f>$H$15*C91</f>
-        <v/>
-      </c>
-      <c r="E91" s="424">
-        <f>(($C$40+(D91*E$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="F91" s="424">
-        <f>(($C$40+(D91*F$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="G91" s="424">
-        <f>(($C$40+(D91*G$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-      <c r="H91" s="424">
-        <f>(($C$40+(D91*H$85)/(1+$C$9)^$H$30)-$C$47)/$C$8</f>
-        <v/>
-      </c>
-    </row>
+      <c r="C91" s="104" t="n"/>
+      <c r="D91" s="101" t="n"/>
+      <c r="E91" s="63" t="n"/>
+      <c r="F91" s="63" t="n"/>
+      <c r="G91" s="63" t="n"/>
+      <c r="H91" s="63" t="n"/>
+    </row>
+    <row r="92"/>
     <row r="93" ht="15.75" customHeight="1" s="381" thickBot="1">
-      <c r="B93" s="389" t="inlineStr">
-        <is>
-          <t>Football field</t>
+      <c r="B93" s="388" t="inlineStr">
+        <is>
+          <t>Football field (chart removed so Excel can open this file)</t>
         </is>
       </c>
       <c r="C93" s="44" t="n"/>
       <c r="D93" s="44" t="n"/>
       <c r="E93" s="44" t="n"/>
     </row>
-    <row r="94">
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>Sources: AI_Operating FCF build; Assumptions_Drivers tax/g/exit; LBO price/shares/debt/cash; Debt_Sweep_AI stack for kd; Strategy_Summary equity check; 52wkHL for market range.</t>
-        </is>
-      </c>
-    </row>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
     <row r="114">
       <c r="B114" s="79" t="n"/>
       <c r="C114" s="80" t="inlineStr">
@@ -26495,39 +24127,33 @@
     <row r="115">
       <c r="B115" s="76" t="inlineStr">
         <is>
-          <t>DCF Value at exit-multiple band (10.9x–14.9x)</t>
-        </is>
-      </c>
-      <c r="C115" s="424">
-        <f>D76</f>
-        <v/>
-      </c>
-      <c r="D115" s="424">
-        <f>E115-C115</f>
-        <v/>
-      </c>
-      <c r="E115" s="439">
-        <f>H81</f>
-        <v/>
+          <t>DCF exit-multiple value / share (cached)</t>
+        </is>
+      </c>
+      <c r="C115" s="390" t="n">
+        <v>8.10863430429332</v>
+      </c>
+      <c r="D115" s="390" t="n">
+        <v>0</v>
+      </c>
+      <c r="E115" s="423" t="n">
+        <v>8.10863430429332</v>
       </c>
     </row>
     <row r="116">
       <c r="B116" s="74" t="inlineStr">
         <is>
-          <t>DCF Value at 1.0%–3.0% Perpetuity Range</t>
-        </is>
-      </c>
-      <c r="C116" s="424">
-        <f>D66</f>
-        <v/>
-      </c>
-      <c r="D116" s="424">
-        <f>E116-C116</f>
-        <v/>
-      </c>
-      <c r="E116" s="439">
-        <f>H71</f>
-        <v/>
+          <t>DCF perpetuity value / share (cached)</t>
+        </is>
+      </c>
+      <c r="C116" s="390" t="n">
+        <v>7.207102552146641</v>
+      </c>
+      <c r="D116" s="390" t="n">
+        <v>0</v>
+      </c>
+      <c r="E116" s="423" t="n">
+        <v>7.207102552146641</v>
       </c>
     </row>
     <row r="117">
@@ -26536,14 +24162,14 @@
           <t>LBO Offer price / share</t>
         </is>
       </c>
-      <c r="C117" s="424">
+      <c r="C117" s="390">
         <f>LBO!H20</f>
         <v/>
       </c>
-      <c r="D117" s="424" t="n">
-        <v>0</v>
-      </c>
-      <c r="E117" s="439">
+      <c r="D117" s="390" t="n">
+        <v>0</v>
+      </c>
+      <c r="E117" s="423">
         <f>LBO!H20</f>
         <v/>
       </c>
@@ -26554,17 +24180,15 @@
           <t>52 Week Market High/Low (GTM)</t>
         </is>
       </c>
-      <c r="C118" s="440">
-        <f>'52wkHL'!E5</f>
-        <v/>
-      </c>
-      <c r="D118" s="440">
+      <c r="C118" s="424" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="D118" s="424">
         <f>E118-C118</f>
         <v/>
       </c>
-      <c r="E118" s="427">
-        <f>'52wkHL'!E4</f>
-        <v/>
+      <c r="E118" s="425" t="n">
+        <v>12.51</v>
       </c>
     </row>
   </sheetData>
@@ -26590,7 +24214,6 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>